<commit_message>
Update white-label plan: apex/www resolved, re-rank levers
Apex/www canonicalisation is done, so drop it as a lever. Master plan
roadmap re-ranked: Phase 0 shrinks to meta-keywords + schema; Tier-A CTR
revamp + hub rebuild becomes the #1 lever (~721k impressions). Redirect
map Data-findings tab reframes apex/www as resolved and notes tiers are
the consolidated single-URL view; excludes chatbot impressions from the
CTR-lift forecast.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UhVChLeNNjFDr6eASTMGhh
</commit_message>
<xml_diff>
--- a/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
+++ b/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
@@ -9142,19 +9142,19 @@
       </c>
       <c r="B4" s="26" t="inlineStr">
         <is>
-          <t>Impressions grew ~46x as programmatic content shipped (13.5k -&gt; 621k per 90 days); clicks only ~1.8x; CTR fell 19.85% -&gt; 0.76%. Relevance/snippet failure at scale, confirmed.</t>
+          <t>Impressions grew ~46x as programmatic content shipped (13.5k -&gt; 621k per 90 days); clicks only ~1.8x; CTR fell 19.85% -&gt; 0.76%. Relevance/snippet failure at scale, confirmed — this (not host duplication) is now the primary problem.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>Apex vs www</t>
+          <t>Apex/www — RESOLVED</t>
         </is>
       </c>
       <c r="B5" s="26" t="inlineStr">
         <is>
-          <t>www 1,365,616 impr @0.94% CTR; apex 1,027,877 impr @0.64%. 87 of 179 white-label paths appear on BOTH hosts, splitting 677,654 impressions. Biggest single lever.</t>
+          <t>Host duplication has been canonicalised to a single host (no longer a lever). The 16-mo export still shows both hosts historically; tiers here are deduped by path, i.e. the consolidated single-URL view. Re-pull GSC in 4-8 weeks to measure the consolidation lift.</t>
         </is>
       </c>
     </row>
@@ -9173,12 +9173,12 @@
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Revamp prize</t>
+          <t>Revamp prize (#1 lever now)</t>
         </is>
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>93 WL pages sit in striking distance (pos&lt;=20, impr&gt;=1000, CTR&lt;1.5%) holding ~721,000 impressions — the Tier-A revamp target.</t>
+          <t>93 WL pages sit in striking distance (pos&lt;=20, impr&gt;=1000, CTR&lt;1.5%) holding ~721,000 impressions — the Tier-A revamp target and, with apex/www done, the single biggest lever. Note: exclude chatbot-query impressions (structurally unconvertible for a voice product) from any CTR-lift forecast.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reverse 6 competitor merges after SERP validation
Live-SERP spot-checks show "X alternative" (roundup intent) and "Trillet
vs X" (head-to-head) are distinct intents, and several Trillet alternative
pages already rank for their term (my-ai-front-desk-alternative #2, vapi
alternative #3, retell white-label converter). Flip those 6 from
REDIRECT to KEEP with the evidence noted; canonical vs-page notes updated.
REDIRECT 15->9, KEEP 138->144. Same-topic dupes unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UhVChLeNNjFDr6eASTMGhh
</commit_message>
<xml_diff>
--- a/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
+++ b/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
@@ -4165,16 +4165,12 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D84" s="12" t="inlineStr">
-        <is>
-          <t>REDIRECT</t>
-        </is>
-      </c>
-      <c r="E84" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/trillet-vs-my-ai-front-desk-comparison-2026</t>
-        </is>
-      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr"/>
       <c r="F84" s="5" t="n">
         <v>13268</v>
       </c>
@@ -4194,7 +4190,7 @@
       </c>
       <c r="K84" s="4" t="inlineStr">
         <is>
-          <t>Duplicate; 301.</t>
+          <t>SERP-validated (keep): ranks #2 for "my ai front desk alternative" — distinct intent from the vs.</t>
         </is>
       </c>
     </row>
@@ -4212,16 +4208,12 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D85" s="12" t="inlineStr">
-        <is>
-          <t>REDIRECT</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/trillet-vs-my-ai-front-desk-comparison-2026</t>
-        </is>
-      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr"/>
       <c r="F85" s="5" t="n">
         <v>4065</v>
       </c>
@@ -4241,7 +4233,7 @@
       </c>
       <c r="K85" s="4" t="inlineStr">
         <is>
-          <t>Duplicate; 301.</t>
+          <t>SERP-validated (keep): distinct white-label angle; differentiate from alternative-2026 (general) and the vs (head-to-head).</t>
         </is>
       </c>
     </row>
@@ -4517,16 +4509,12 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D92" s="12" t="inlineStr">
-        <is>
-          <t>REDIRECT</t>
-        </is>
-      </c>
-      <c r="E92" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/trillet-vs-retell-vs-vapi-comparison</t>
-        </is>
-      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr"/>
       <c r="F92" s="5" t="n">
         <v>15338</v>
       </c>
@@ -4546,7 +4534,7 @@
       </c>
       <c r="K92" s="4" t="inlineStr">
         <is>
-          <t>301 to canonical vs.</t>
+          <t>SERP-validated (keep): owns the converting "retell ai white label" niche (3.35% CTR); distinct intent from the head-to-head vs.</t>
         </is>
       </c>
     </row>
@@ -4564,16 +4552,12 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D93" s="12" t="inlineStr">
-        <is>
-          <t>REDIRECT</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/trillet-vs-smith-ai-comparison-2026</t>
-        </is>
-      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr"/>
       <c r="F93" s="5" t="n">
         <v>14244</v>
       </c>
@@ -4593,7 +4577,7 @@
       </c>
       <c r="K93" s="4" t="inlineStr">
         <is>
-          <t>Duplicate; 301.</t>
+          <t>SERP-validated (keep): "smith ai alternative" is roundup intent, distinct from the head-to-head vs.</t>
         </is>
       </c>
     </row>
@@ -4654,16 +4638,12 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D95" s="12" t="inlineStr">
-        <is>
-          <t>REDIRECT</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/synthflow-vs-trillet-comparison</t>
-        </is>
-      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr"/>
       <c r="F95" s="5" t="n">
         <v>8265</v>
       </c>
@@ -4683,7 +4663,7 @@
       </c>
       <c r="K95" s="4" t="inlineStr">
         <is>
-          <t>Duplicate; 301.</t>
+          <t>SERP-validated (keep): distinct agency-angle content; co-ranks only on the brand term. Differentiate from the vs.</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4706,7 @@
       </c>
       <c r="K96" s="4" t="inlineStr">
         <is>
-          <t>Canonical Synthflow page.</t>
+          <t>Canonical head-to-head. synthflow-alternative-for-agencies has distinct content and is KEPT (SERP-validated).</t>
         </is>
       </c>
     </row>
@@ -5113,7 +5093,7 @@
       </c>
       <c r="K105" s="4" t="inlineStr">
         <is>
-          <t>Canonical My AI Front Desk page.</t>
+          <t>Canonical head-to-head. The two MAFD alternative pages serve different intent and are KEPT (SERP-validated), not merged here.</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5136,7 @@
       </c>
       <c r="K106" s="4" t="inlineStr">
         <is>
-          <t>Canonical Retell/Vapi comparison.</t>
+          <t>Canonical head-to-head. The Retell/Vapi white-label "alternative" pages own distinct intent and are KEPT (SERP-validated).</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5222,7 @@
       </c>
       <c r="K108" s="4" t="inlineStr">
         <is>
-          <t>Canonical Smith.ai page.</t>
+          <t>Canonical head-to-head. smith-ai-alternative-2026 owns roundup intent and is KEPT (SERP-validated).</t>
         </is>
       </c>
     </row>
@@ -5303,16 +5283,12 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D110" s="12" t="inlineStr">
-        <is>
-          <t>REDIRECT</t>
-        </is>
-      </c>
-      <c r="E110" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/trillet-vs-retell-vs-vapi-comparison</t>
-        </is>
-      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr"/>
       <c r="F110" s="5" t="n">
         <v>3834</v>
       </c>
@@ -5332,7 +5308,7 @@
       </c>
       <c r="K110" s="4" t="inlineStr">
         <is>
-          <t>Thin agency-alt; 301 to canonical vs.</t>
+          <t>SERP-validated (keep): ranks p1 (#3) for "vapi alternative for agencies" — roundup intent, distinct from the vs.</t>
         </is>
       </c>
     </row>
@@ -8903,7 +8879,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
@@ -8923,7 +8899,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Add query-overlap data to redirect map + 3 survivor fixes
Ran the GSC query-overlap check on all 24 merge/redirect pairs. Low exact
overlap is largely a Google-dedup artifact; shared-query evidence confirms
same intent, so merges hold. Data surfaced 3 survivor/direction fixes:
reverse voice-vs-text canonical to the 75-query page; reframe (not redirect)
the 96-query how-to-start-ai-chatbot-agency to voice; flag wrapper/native
survivor (13 vs 2 queries). Overlap % + verdict added as columns; raw
results archived.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UhVChLeNNjFDr6eASTMGhh
</commit_message>
<xml_diff>
--- a/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
+++ b/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Data findings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Redirect map'!$A$1:$K$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Redirect map'!$A$1:$M$191</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -98,12 +98,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFE0FB"/>
+        <fgColor rgb="00E4D4F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E4D4F0"/>
+        <fgColor rgb="00CFE0FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,11 +183,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K191"/>
+  <dimension ref="A1:M191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -573,7 +573,9 @@
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="58" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="58" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,6 +631,16 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Overlap %</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Overlap verdict</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Reason / note</t>
         </is>
       </c>
@@ -670,7 +682,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Rebuild as the cluster hub (title/H1/subhead, SoftwareApplication+Offer schema, remove meta-kw, links to all spokes).</t>
         </is>
@@ -713,7 +727,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr"/>
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Canonical pricing target. Point all WL-pricing blogs here.</t>
         </is>
@@ -756,7 +772,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Rebuild as partner-program hub (Reseller/OEM/Referral/Agency tiers, benefits, apply CTA).</t>
         </is>
@@ -791,7 +809,9 @@
           <t>n/a (build)</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>NEW integrations directory hub.</t>
         </is>
@@ -826,7 +846,9 @@
           <t>n/a (build)</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>NEW canonical GoHighLevel landing page (consolidates GHL posts as spokes).</t>
         </is>
@@ -861,7 +883,9 @@
           <t>n/a (build)</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>NEW AI Voice Agency Academy hub — organises the ~45 business posts into a learning path.</t>
         </is>
@@ -896,7 +920,9 @@
           <t>n/a (build)</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>NEW white-label-by-industry index — links the ~25 vertical posts + their /receptionist/industries counterparts.</t>
         </is>
@@ -931,7 +957,9 @@
           <t>n/a (build)</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>NEW compare &amp; alternatives index — links all vs/alternative pages, one per competitor.</t>
         </is>
@@ -966,7 +994,9 @@
           <t>n/a (build)</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>NEW /reviews social-proof hub (Review schema).</t>
         </is>
@@ -1009,7 +1039,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1052,7 +1084,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1072,9 +1106,9 @@
           <t>2 · Agency Academy</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>CANONICAL</t>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr"/>
@@ -1095,9 +1129,11 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>Canonical "how to start a voice AI agency" (Academy entry).</t>
+      <c r="K13" s="5" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Distinct 60-day-plan format (only 2 queries). Pair with the reframed how-to-start page; consider merging later.</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1174,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -1181,7 +1219,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1224,7 +1264,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1267,7 +1309,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1310,7 +1354,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1353,7 +1399,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1396,7 +1444,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1443,7 +1493,17 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>Chatbot; 301 to voice canvas.</t>
         </is>
@@ -1486,7 +1546,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1529,7 +1591,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1572,7 +1636,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1615,7 +1681,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="K25" s="5" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -1658,7 +1726,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="K26" s="5" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -1701,7 +1771,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="K27" s="5" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
+      <c r="M27" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -1744,7 +1816,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="K28" s="5" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1787,7 +1861,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="K29" s="5" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1830,7 +1906,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="K30" s="5" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr"/>
+      <c r="M30" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1873,7 +1951,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="K31" s="5" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1920,7 +2000,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
         <is>
           <t>Fold into the canonical pricing guide; 301.</t>
         </is>
@@ -1963,7 +2053,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K33" s="4" t="inlineStr">
+      <c r="K33" s="5" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr"/>
+      <c r="M33" s="4" t="inlineStr">
         <is>
           <t>Canonical agency-economics post.</t>
         </is>
@@ -2006,7 +2098,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K34" s="4" t="inlineStr">
+      <c r="K34" s="5" t="inlineStr"/>
+      <c r="L34" s="4" t="inlineStr"/>
+      <c r="M34" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2041,7 +2135,9 @@
           <t>C · interlink/prune (no traffic)</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="K35" s="5" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2084,7 +2180,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="K36" s="5" t="inlineStr"/>
+      <c r="L36" s="4" t="inlineStr"/>
+      <c r="M36" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2127,7 +2225,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="K37" s="5" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2170,7 +2270,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="K38" s="5" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr"/>
+      <c r="M38" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -2217,7 +2319,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr">
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>10.7</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
         <is>
           <t>Fold into canonical roundup; 301.</t>
         </is>
@@ -2264,7 +2376,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K40" s="4" t="inlineStr">
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
         <is>
           <t>Chatbot-framed; 301 to voice roundup.</t>
         </is>
@@ -2311,7 +2433,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K41" s="4" t="inlineStr">
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
         <is>
           <t>Fold into canonical roundup; 301.</t>
         </is>
@@ -2354,7 +2486,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K42" s="4" t="inlineStr">
+      <c r="K42" s="5" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr"/>
+      <c r="M42" s="4" t="inlineStr">
         <is>
           <t>Distinct build-vs-buy angle; keep as canonical build-vs-buy.</t>
         </is>
@@ -2397,7 +2531,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K43" s="4" t="inlineStr">
+      <c r="K43" s="5" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
+      <c r="M43" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2440,7 +2576,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K44" s="4" t="inlineStr">
+      <c r="K44" s="5" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr"/>
+      <c r="M44" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2483,7 +2621,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K45" s="4" t="inlineStr">
+      <c r="K45" s="5" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
+      <c r="M45" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2526,7 +2666,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K46" s="4" t="inlineStr">
+      <c r="K46" s="5" t="inlineStr"/>
+      <c r="L46" s="4" t="inlineStr"/>
+      <c r="M46" s="4" t="inlineStr">
         <is>
           <t>Distinct "cheapest" price intent; keep, link to hub + pricing guide.</t>
         </is>
@@ -2569,7 +2711,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K47" s="4" t="inlineStr">
+      <c r="K47" s="5" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
+      <c r="M47" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2612,7 +2756,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K48" s="4" t="inlineStr">
+      <c r="K48" s="5" t="inlineStr"/>
+      <c r="L48" s="4" t="inlineStr"/>
+      <c r="M48" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2655,7 +2801,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K49" s="4" t="inlineStr">
+      <c r="K49" s="5" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
+      <c r="M49" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2698,7 +2846,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K50" s="4" t="inlineStr">
+      <c r="K50" s="5" t="inlineStr"/>
+      <c r="L50" s="4" t="inlineStr"/>
+      <c r="M50" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2741,7 +2891,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K51" s="4" t="inlineStr">
+      <c r="K51" s="5" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr"/>
+      <c r="M51" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2784,7 +2936,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K52" s="4" t="inlineStr">
+      <c r="K52" s="5" t="inlineStr"/>
+      <c r="L52" s="4" t="inlineStr"/>
+      <c r="M52" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2831,7 +2985,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K53" s="4" t="inlineStr">
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M53" s="4" t="inlineStr">
         <is>
           <t>Fold into canonical roundup; 301.</t>
         </is>
@@ -2874,7 +3038,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K54" s="4" t="inlineStr">
+      <c r="K54" s="5" t="inlineStr"/>
+      <c r="L54" s="4" t="inlineStr"/>
+      <c r="M54" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2917,7 +3083,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K55" s="4" t="inlineStr">
+      <c r="K55" s="5" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr"/>
+      <c r="M55" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2960,7 +3128,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K56" s="4" t="inlineStr">
+      <c r="K56" s="5" t="inlineStr"/>
+      <c r="L56" s="4" t="inlineStr"/>
+      <c r="M56" s="4" t="inlineStr">
         <is>
           <t>Distinct how-to; keep as GHL spoke.</t>
         </is>
@@ -3007,7 +3177,17 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K57" s="4" t="inlineStr">
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>33.3</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM - review shared</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
         <is>
           <t>Same intent; merge + 301.</t>
         </is>
@@ -3050,7 +3230,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K58" s="4" t="inlineStr">
+      <c r="K58" s="5" t="inlineStr"/>
+      <c r="L58" s="4" t="inlineStr"/>
+      <c r="M58" s="4" t="inlineStr">
         <is>
           <t>Distinct angle; keep as GHL spoke.</t>
         </is>
@@ -3097,7 +3279,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K59" s="4" t="inlineStr">
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="inlineStr">
         <is>
           <t>Fold into the new GHL landing page; 301.</t>
         </is>
@@ -3144,7 +3336,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K60" s="4" t="inlineStr">
+      <c r="K60" s="5" t="inlineStr">
+        <is>
+          <t>25.6</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM - review shared</t>
+        </is>
+      </c>
+      <c r="M60" s="4" t="inlineStr">
         <is>
           <t>Same intent; merge + 301.</t>
         </is>
@@ -3187,7 +3389,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K61" s="4" t="inlineStr">
+      <c r="K61" s="5" t="inlineStr"/>
+      <c r="L61" s="4" t="inlineStr"/>
+      <c r="M61" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -3230,7 +3434,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K62" s="4" t="inlineStr">
+      <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="4" t="inlineStr"/>
+      <c r="M62" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3269,7 +3475,17 @@
           <t>C · interlink/prune (no traffic)</t>
         </is>
       </c>
-      <c r="K63" s="4" t="inlineStr">
+      <c r="K63" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>SOURCE HAS NO QUERIES - safe to redirect</t>
+        </is>
+      </c>
+      <c r="M63" s="4" t="inlineStr">
         <is>
           <t>Chatbot definitional; 301 to voice.</t>
         </is>
@@ -3312,7 +3528,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K64" s="4" t="inlineStr">
+      <c r="K64" s="5" t="inlineStr"/>
+      <c r="L64" s="4" t="inlineStr"/>
+      <c r="M64" s="4" t="inlineStr">
         <is>
           <t>Distinct cost-to-start intent; keep.</t>
         </is>
@@ -3359,7 +3577,17 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K65" s="4" t="inlineStr">
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L65" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M65" s="4" t="inlineStr">
         <is>
           <t>Same intent; merge + 301.</t>
         </is>
@@ -3402,7 +3630,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K66" s="4" t="inlineStr">
+      <c r="K66" s="5" t="inlineStr"/>
+      <c r="L66" s="4" t="inlineStr"/>
+      <c r="M66" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3445,7 +3675,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K67" s="4" t="inlineStr">
+      <c r="K67" s="5" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
+      <c r="M67" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3492,7 +3724,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K68" s="4" t="inlineStr">
+      <c r="K68" s="5" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="L68" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M68" s="4" t="inlineStr">
         <is>
           <t>Chatbot; 301 to voice features checklist.</t>
         </is>
@@ -3535,7 +3777,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K69" s="4" t="inlineStr">
+      <c r="K69" s="5" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr"/>
+      <c r="M69" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3578,7 +3822,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K70" s="4" t="inlineStr">
+      <c r="K70" s="5" t="inlineStr"/>
+      <c r="L70" s="4" t="inlineStr"/>
+      <c r="M70" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3621,7 +3867,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K71" s="4" t="inlineStr">
+      <c r="K71" s="5" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
+      <c r="M71" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3641,16 +3889,12 @@
           <t>2 · Agency Academy</t>
         </is>
       </c>
-      <c r="D72" s="12" t="inlineStr">
-        <is>
-          <t>REDIRECT</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/60-day-ai-voice-agency-launch-plan</t>
-        </is>
-      </c>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>REFRAME</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr"/>
       <c r="F72" s="5" t="n">
         <v>25911</v>
       </c>
@@ -3668,9 +3912,19 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K72" s="4" t="inlineStr">
-        <is>
-          <t>Chatbot-framed start; 301 to voice launch plan.</t>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="L72" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M72" s="4" t="inlineStr">
+        <is>
+          <t>GSC: 96 queries — too much traffic to redirect. Rewrite to voice framing ("how to start a voice AI agency") and keep the URL as a primary start guide.</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3965,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K73" s="4" t="inlineStr">
+      <c r="K73" s="5" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+      <c r="M73" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3754,7 +4010,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K74" s="4" t="inlineStr">
+      <c r="K74" s="5" t="inlineStr"/>
+      <c r="L74" s="4" t="inlineStr"/>
+      <c r="M74" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -3797,7 +4055,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K75" s="4" t="inlineStr">
+      <c r="K75" s="5" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr"/>
+      <c r="M75" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -3840,7 +4100,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K76" s="4" t="inlineStr">
+      <c r="K76" s="5" t="inlineStr"/>
+      <c r="L76" s="4" t="inlineStr"/>
+      <c r="M76" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -3883,7 +4145,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K77" s="4" t="inlineStr">
+      <c r="K77" s="5" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
+      <c r="M77" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3926,7 +4190,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K78" s="4" t="inlineStr">
+      <c r="K78" s="5" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr"/>
+      <c r="M78" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -3969,7 +4235,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K79" s="4" t="inlineStr">
+      <c r="K79" s="5" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+      <c r="M79" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -4012,7 +4280,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K80" s="4" t="inlineStr">
+      <c r="K80" s="5" t="inlineStr"/>
+      <c r="L80" s="4" t="inlineStr"/>
+      <c r="M80" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4055,7 +4325,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K81" s="4" t="inlineStr">
+      <c r="K81" s="5" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr"/>
+      <c r="M81" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4102,7 +4374,17 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K82" s="4" t="inlineStr">
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L82" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M82" s="4" t="inlineStr">
         <is>
           <t>Same intent; merge as a section + 301.</t>
         </is>
@@ -4145,7 +4427,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K83" s="4" t="inlineStr">
+      <c r="K83" s="5" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr"/>
+      <c r="M83" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -4188,7 +4472,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K84" s="4" t="inlineStr">
+      <c r="K84" s="5" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr"/>
+      <c r="M84" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): ranks #2 for "my ai front desk alternative" — distinct intent from the vs.</t>
         </is>
@@ -4231,7 +4517,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K85" s="4" t="inlineStr">
+      <c r="K85" s="5" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+      <c r="M85" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): distinct white-label angle; differentiate from alternative-2026 (general) and the vs (head-to-head).</t>
         </is>
@@ -4274,7 +4562,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K86" s="4" t="inlineStr">
+      <c r="K86" s="5" t="inlineStr"/>
+      <c r="L86" s="4" t="inlineStr"/>
+      <c r="M86" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -4317,7 +4607,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K87" s="4" t="inlineStr">
+      <c r="K87" s="5" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+      <c r="M87" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -4360,7 +4652,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K88" s="4" t="inlineStr">
+      <c r="K88" s="5" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
+      <c r="M88" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4403,7 +4697,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K89" s="4" t="inlineStr">
+      <c r="K89" s="5" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+      <c r="M89" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4446,7 +4742,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K90" s="4" t="inlineStr">
+      <c r="K90" s="5" t="inlineStr"/>
+      <c r="L90" s="4" t="inlineStr"/>
+      <c r="M90" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4489,7 +4787,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K91" s="4" t="inlineStr">
+      <c r="K91" s="5" t="inlineStr"/>
+      <c r="L91" s="4" t="inlineStr"/>
+      <c r="M91" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -4532,7 +4832,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K92" s="4" t="inlineStr">
+      <c r="K92" s="5" t="inlineStr"/>
+      <c r="L92" s="4" t="inlineStr"/>
+      <c r="M92" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): owns the converting "retell ai white label" niche (3.35% CTR); distinct intent from the head-to-head vs.</t>
         </is>
@@ -4575,7 +4877,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K93" s="4" t="inlineStr">
+      <c r="K93" s="5" t="inlineStr"/>
+      <c r="L93" s="4" t="inlineStr"/>
+      <c r="M93" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): "smith ai alternative" is roundup intent, distinct from the head-to-head vs.</t>
         </is>
@@ -4618,7 +4922,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K94" s="4" t="inlineStr">
+      <c r="K94" s="5" t="inlineStr"/>
+      <c r="L94" s="4" t="inlineStr"/>
+      <c r="M94" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4661,7 +4967,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K95" s="4" t="inlineStr">
+      <c r="K95" s="5" t="inlineStr"/>
+      <c r="L95" s="4" t="inlineStr"/>
+      <c r="M95" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): distinct agency-angle content; co-ranks only on the brand term. Differentiate from the vs.</t>
         </is>
@@ -4704,7 +5012,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K96" s="4" t="inlineStr">
+      <c r="K96" s="5" t="inlineStr"/>
+      <c r="L96" s="4" t="inlineStr"/>
+      <c r="M96" s="4" t="inlineStr">
         <is>
           <t>Canonical head-to-head. synthflow-alternative-for-agencies has distinct content and is KEPT (SERP-validated).</t>
         </is>
@@ -4747,7 +5057,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K97" s="4" t="inlineStr">
+      <c r="K97" s="5" t="inlineStr"/>
+      <c r="L97" s="4" t="inlineStr"/>
+      <c r="M97" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4790,7 +5102,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K98" s="4" t="inlineStr">
+      <c r="K98" s="5" t="inlineStr"/>
+      <c r="L98" s="4" t="inlineStr"/>
+      <c r="M98" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4810,7 +5124,7 @@
           <t>2 · Agency Academy</t>
         </is>
       </c>
-      <c r="D99" s="14" t="inlineStr">
+      <c r="D99" s="15" t="inlineStr">
         <is>
           <t>REVAMP</t>
         </is>
@@ -4833,7 +5147,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K99" s="4" t="inlineStr">
+      <c r="K99" s="5" t="inlineStr"/>
+      <c r="L99" s="4" t="inlineStr"/>
+      <c r="M99" s="4" t="inlineStr">
         <is>
           <t>Canonical "best white-label voice AI" roundup. Rewrite as honest named comparison + current data.</t>
         </is>
@@ -4876,7 +5192,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K100" s="4" t="inlineStr">
+      <c r="K100" s="5" t="inlineStr"/>
+      <c r="L100" s="4" t="inlineStr"/>
+      <c r="M100" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4919,7 +5237,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K101" s="4" t="inlineStr">
+      <c r="K101" s="5" t="inlineStr"/>
+      <c r="L101" s="4" t="inlineStr"/>
+      <c r="M101" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4962,7 +5282,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K102" s="4" t="inlineStr">
+      <c r="K102" s="5" t="inlineStr"/>
+      <c r="L102" s="4" t="inlineStr"/>
+      <c r="M102" s="4" t="inlineStr">
         <is>
           <t>Canonical "GHL native vs Trillet" comparison.</t>
         </is>
@@ -5005,7 +5327,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K103" s="4" t="inlineStr">
+      <c r="K103" s="5" t="inlineStr"/>
+      <c r="L103" s="4" t="inlineStr"/>
+      <c r="M103" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5048,7 +5372,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K104" s="4" t="inlineStr">
+      <c r="K104" s="5" t="inlineStr"/>
+      <c r="L104" s="4" t="inlineStr"/>
+      <c r="M104" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5091,7 +5417,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K105" s="4" t="inlineStr">
+      <c r="K105" s="5" t="inlineStr"/>
+      <c r="L105" s="4" t="inlineStr"/>
+      <c r="M105" s="4" t="inlineStr">
         <is>
           <t>Canonical head-to-head. The two MAFD alternative pages serve different intent and are KEPT (SERP-validated), not merged here.</t>
         </is>
@@ -5134,7 +5462,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K106" s="4" t="inlineStr">
+      <c r="K106" s="5" t="inlineStr"/>
+      <c r="L106" s="4" t="inlineStr"/>
+      <c r="M106" s="4" t="inlineStr">
         <is>
           <t>Canonical head-to-head. The Retell/Vapi white-label "alternative" pages own distinct intent and are KEPT (SERP-validated).</t>
         </is>
@@ -5177,7 +5507,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K107" s="4" t="inlineStr">
+      <c r="K107" s="5" t="inlineStr"/>
+      <c r="L107" s="4" t="inlineStr"/>
+      <c r="M107" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5220,7 +5552,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K108" s="4" t="inlineStr">
+      <c r="K108" s="5" t="inlineStr"/>
+      <c r="L108" s="4" t="inlineStr"/>
+      <c r="M108" s="4" t="inlineStr">
         <is>
           <t>Canonical head-to-head. smith-ai-alternative-2026 owns roundup intent and is KEPT (SERP-validated).</t>
         </is>
@@ -5263,7 +5597,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K109" s="4" t="inlineStr">
+      <c r="K109" s="5" t="inlineStr"/>
+      <c r="L109" s="4" t="inlineStr"/>
+      <c r="M109" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5306,7 +5642,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K110" s="4" t="inlineStr">
+      <c r="K110" s="5" t="inlineStr"/>
+      <c r="L110" s="4" t="inlineStr"/>
+      <c r="M110" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): ranks p1 (#3) for "vapi alternative for agencies" — roundup intent, distinct from the vs.</t>
         </is>
@@ -5349,7 +5687,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K111" s="4" t="inlineStr">
+      <c r="K111" s="5" t="inlineStr"/>
+      <c r="L111" s="4" t="inlineStr"/>
+      <c r="M111" s="4" t="inlineStr">
         <is>
           <t>Distinct compliance angle (the wedge); keep.</t>
         </is>
@@ -5392,7 +5732,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K112" s="4" t="inlineStr">
+      <c r="K112" s="5" t="inlineStr"/>
+      <c r="L112" s="4" t="inlineStr"/>
+      <c r="M112" s="4" t="inlineStr">
         <is>
           <t>Distinct: Vapi own WL options; keep.</t>
         </is>
@@ -5435,7 +5777,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K113" s="4" t="inlineStr">
+      <c r="K113" s="5" t="inlineStr"/>
+      <c r="L113" s="4" t="inlineStr"/>
+      <c r="M113" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5478,7 +5822,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K114" s="4" t="inlineStr">
+      <c r="K114" s="5" t="inlineStr"/>
+      <c r="L114" s="4" t="inlineStr"/>
+      <c r="M114" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -5521,7 +5867,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K115" s="4" t="inlineStr">
+      <c r="K115" s="5" t="inlineStr"/>
+      <c r="L115" s="4" t="inlineStr"/>
+      <c r="M115" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -5564,7 +5912,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K116" s="4" t="inlineStr">
+      <c r="K116" s="5" t="inlineStr"/>
+      <c r="L116" s="4" t="inlineStr"/>
+      <c r="M116" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -5607,7 +5957,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K117" s="4" t="inlineStr">
+      <c r="K117" s="5" t="inlineStr"/>
+      <c r="L117" s="4" t="inlineStr"/>
+      <c r="M117" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -5650,7 +6002,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K118" s="4" t="inlineStr">
+      <c r="K118" s="5" t="inlineStr"/>
+      <c r="L118" s="4" t="inlineStr"/>
+      <c r="M118" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -5693,7 +6047,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K119" s="4" t="inlineStr">
+      <c r="K119" s="5" t="inlineStr"/>
+      <c r="L119" s="4" t="inlineStr"/>
+      <c r="M119" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -5736,7 +6092,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K120" s="4" t="inlineStr">
+      <c r="K120" s="5" t="inlineStr"/>
+      <c r="L120" s="4" t="inlineStr"/>
+      <c r="M120" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5756,7 +6114,7 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D121" s="15" t="inlineStr">
+      <c r="D121" s="14" t="inlineStr">
         <is>
           <t>REFRAME</t>
         </is>
@@ -5771,7 +6129,9 @@
           <t>C · interlink/prune (no traffic)</t>
         </is>
       </c>
-      <c r="K121" s="4" t="inlineStr">
+      <c r="K121" s="5" t="inlineStr"/>
+      <c r="L121" s="4" t="inlineStr"/>
+      <c r="M121" s="4" t="inlineStr">
         <is>
           <t>KEEP but sharpen "sell voice, not chat"; the chatbot-&gt;voice converter.</t>
         </is>
@@ -5814,7 +6174,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K122" s="4" t="inlineStr">
+      <c r="K122" s="5" t="inlineStr"/>
+      <c r="L122" s="4" t="inlineStr"/>
+      <c r="M122" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -5857,7 +6219,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K123" s="4" t="inlineStr">
+      <c r="K123" s="5" t="inlineStr"/>
+      <c r="L123" s="4" t="inlineStr"/>
+      <c r="M123" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -5900,7 +6264,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K124" s="4" t="inlineStr">
+      <c r="K124" s="5" t="inlineStr"/>
+      <c r="L124" s="4" t="inlineStr"/>
+      <c r="M124" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -5943,7 +6309,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K125" s="4" t="inlineStr">
+      <c r="K125" s="5" t="inlineStr"/>
+      <c r="L125" s="4" t="inlineStr"/>
+      <c r="M125" s="4" t="inlineStr">
         <is>
           <t>Distinct ROI tool; keep.</t>
         </is>
@@ -5982,7 +6350,17 @@
           <t>C · interlink/prune (no traffic)</t>
         </is>
       </c>
-      <c r="K126" s="4" t="inlineStr">
+      <c r="K126" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L126" s="4" t="inlineStr">
+        <is>
+          <t>SOURCE HAS NO QUERIES - safe to redirect</t>
+        </is>
+      </c>
+      <c r="M126" s="4" t="inlineStr">
         <is>
           <t>Merge + 301.</t>
         </is>
@@ -6025,7 +6403,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K127" s="4" t="inlineStr">
+      <c r="K127" s="5" t="inlineStr"/>
+      <c r="L127" s="4" t="inlineStr"/>
+      <c r="M127" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -6060,7 +6440,9 @@
           <t>C · interlink/prune (no traffic)</t>
         </is>
       </c>
-      <c r="K128" s="4" t="inlineStr">
+      <c r="K128" s="5" t="inlineStr"/>
+      <c r="L128" s="4" t="inlineStr"/>
+      <c r="M128" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -6103,7 +6485,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K129" s="4" t="inlineStr">
+      <c r="K129" s="5" t="inlineStr"/>
+      <c r="L129" s="4" t="inlineStr"/>
+      <c r="M129" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6146,7 +6530,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K130" s="4" t="inlineStr">
+      <c r="K130" s="5" t="inlineStr"/>
+      <c r="L130" s="4" t="inlineStr"/>
+      <c r="M130" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6189,7 +6575,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K131" s="4" t="inlineStr">
+      <c r="K131" s="5" t="inlineStr"/>
+      <c r="L131" s="4" t="inlineStr"/>
+      <c r="M131" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6232,7 +6620,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K132" s="4" t="inlineStr">
+      <c r="K132" s="5" t="inlineStr"/>
+      <c r="L132" s="4" t="inlineStr"/>
+      <c r="M132" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6275,7 +6665,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K133" s="4" t="inlineStr">
+      <c r="K133" s="5" t="inlineStr"/>
+      <c r="L133" s="4" t="inlineStr"/>
+      <c r="M133" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6318,7 +6710,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K134" s="4" t="inlineStr">
+      <c r="K134" s="5" t="inlineStr"/>
+      <c r="L134" s="4" t="inlineStr"/>
+      <c r="M134" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6361,7 +6755,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K135" s="4" t="inlineStr">
+      <c r="K135" s="5" t="inlineStr"/>
+      <c r="L135" s="4" t="inlineStr"/>
+      <c r="M135" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6404,7 +6800,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K136" s="4" t="inlineStr">
+      <c r="K136" s="5" t="inlineStr"/>
+      <c r="L136" s="4" t="inlineStr"/>
+      <c r="M136" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6447,7 +6845,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K137" s="4" t="inlineStr">
+      <c r="K137" s="5" t="inlineStr"/>
+      <c r="L137" s="4" t="inlineStr"/>
+      <c r="M137" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6490,7 +6890,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K138" s="4" t="inlineStr">
+      <c r="K138" s="5" t="inlineStr"/>
+      <c r="L138" s="4" t="inlineStr"/>
+      <c r="M138" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6533,7 +6935,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K139" s="4" t="inlineStr">
+      <c r="K139" s="5" t="inlineStr"/>
+      <c r="L139" s="4" t="inlineStr"/>
+      <c r="M139" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -6576,7 +6980,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K140" s="4" t="inlineStr">
+      <c r="K140" s="5" t="inlineStr"/>
+      <c r="L140" s="4" t="inlineStr"/>
+      <c r="M140" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -6619,7 +7025,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K141" s="4" t="inlineStr">
+      <c r="K141" s="5" t="inlineStr"/>
+      <c r="L141" s="4" t="inlineStr"/>
+      <c r="M141" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -6662,7 +7070,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K142" s="4" t="inlineStr">
+      <c r="K142" s="5" t="inlineStr"/>
+      <c r="L142" s="4" t="inlineStr"/>
+      <c r="M142" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -6705,7 +7115,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K143" s="4" t="inlineStr">
+      <c r="K143" s="5" t="inlineStr"/>
+      <c r="L143" s="4" t="inlineStr"/>
+      <c r="M143" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -6748,7 +7160,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K144" s="4" t="inlineStr">
+      <c r="K144" s="5" t="inlineStr"/>
+      <c r="L144" s="4" t="inlineStr"/>
+      <c r="M144" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -6775,7 +7189,7 @@
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>/blogs/voice-first-vs-chat-first-platforms</t>
+          <t>/blogs/voice-ai-vs-text-chatbot-comparison</t>
         </is>
       </c>
       <c r="F145" s="5" t="n">
@@ -6795,7 +7209,17 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K145" s="4" t="inlineStr">
+      <c r="K145" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L145" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M145" s="4" t="inlineStr">
         <is>
           <t>Merge + 301.</t>
         </is>
@@ -6815,16 +7239,12 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D146" s="13" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
-      <c r="E146" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/voice-first-vs-chat-first-platforms</t>
-        </is>
-      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>CANONICAL</t>
+        </is>
+      </c>
+      <c r="E146" s="4" t="inlineStr"/>
       <c r="F146" s="5" t="n">
         <v>8335</v>
       </c>
@@ -6842,9 +7262,19 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K146" s="4" t="inlineStr">
-        <is>
-          <t>Merge + 301.</t>
+      <c r="K146" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L146" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M146" s="4" t="inlineStr">
+        <is>
+          <t>GSC-validated survivor: 75 queries vs 21 on the alternative. Canonical voice-vs-text post.</t>
         </is>
       </c>
     </row>
@@ -6862,7 +7292,7 @@
           <t>5 · Pricing &amp; economics</t>
         </is>
       </c>
-      <c r="D147" s="14" t="inlineStr">
+      <c r="D147" s="15" t="inlineStr">
         <is>
           <t>REVAMP</t>
         </is>
@@ -6885,7 +7315,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K147" s="4" t="inlineStr">
+      <c r="K147" s="5" t="inlineStr"/>
+      <c r="L147" s="4" t="inlineStr"/>
+      <c r="M147" s="4" t="inlineStr">
         <is>
           <t>Canonical WL-pricing GUIDE. 46k impressions @0.06% CTR — rewrite title/meta/snippet, add table + CTA to /whitelabel/pricing.</t>
         </is>
@@ -6928,7 +7360,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K148" s="4" t="inlineStr">
+      <c r="K148" s="5" t="inlineStr"/>
+      <c r="L148" s="4" t="inlineStr"/>
+      <c r="M148" s="4" t="inlineStr">
         <is>
           <t>Canonical wrapper-vs-native (the "we own the stack" differentiator).</t>
         </is>
@@ -6948,12 +7382,16 @@
           <t>4 · Compare</t>
         </is>
       </c>
-      <c r="D149" s="3" t="inlineStr">
-        <is>
-          <t>CANONICAL</t>
-        </is>
-      </c>
-      <c r="E149" s="4" t="inlineStr"/>
+      <c r="D149" s="13" t="inlineStr">
+        <is>
+          <t>MERGE</t>
+        </is>
+      </c>
+      <c r="E149" s="4" t="inlineStr">
+        <is>
+          <t>/blogs/voice-ai-vs-text-chatbot-comparison</t>
+        </is>
+      </c>
       <c r="F149" s="5" t="n">
         <v>2149</v>
       </c>
@@ -6971,9 +7409,11 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K149" s="4" t="inlineStr">
-        <is>
-          <t>Canonical voice-vs-text positioning post.</t>
+      <c r="K149" s="5" t="inlineStr"/>
+      <c r="L149" s="4" t="inlineStr"/>
+      <c r="M149" s="4" t="inlineStr">
+        <is>
+          <t>Fewer queries (21 vs 75); merge into the stronger page + 301.</t>
         </is>
       </c>
     </row>
@@ -7014,7 +7454,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K150" s="4" t="inlineStr">
+      <c r="K150" s="5" t="inlineStr"/>
+      <c r="L150" s="4" t="inlineStr"/>
+      <c r="M150" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7057,7 +7499,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K151" s="4" t="inlineStr">
+      <c r="K151" s="5" t="inlineStr"/>
+      <c r="L151" s="4" t="inlineStr"/>
+      <c r="M151" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7100,7 +7544,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K152" s="4" t="inlineStr">
+      <c r="K152" s="5" t="inlineStr"/>
+      <c r="L152" s="4" t="inlineStr"/>
+      <c r="M152" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7143,7 +7589,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K153" s="4" t="inlineStr">
+      <c r="K153" s="5" t="inlineStr"/>
+      <c r="L153" s="4" t="inlineStr"/>
+      <c r="M153" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7186,7 +7634,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K154" s="4" t="inlineStr">
+      <c r="K154" s="5" t="inlineStr"/>
+      <c r="L154" s="4" t="inlineStr"/>
+      <c r="M154" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7233,7 +7683,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K155" s="4" t="inlineStr">
+      <c r="K155" s="5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L155" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M155" s="4" t="inlineStr">
         <is>
           <t>Chatbot definitional; 301 to voice.</t>
         </is>
@@ -7276,7 +7736,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K156" s="4" t="inlineStr">
+      <c r="K156" s="5" t="inlineStr"/>
+      <c r="L156" s="4" t="inlineStr"/>
+      <c r="M156" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -7319,7 +7781,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K157" s="4" t="inlineStr">
+      <c r="K157" s="5" t="inlineStr"/>
+      <c r="L157" s="4" t="inlineStr"/>
+      <c r="M157" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -7362,7 +7826,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K158" s="4" t="inlineStr">
+      <c r="K158" s="5" t="inlineStr"/>
+      <c r="L158" s="4" t="inlineStr"/>
+      <c r="M158" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -7405,7 +7871,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K159" s="4" t="inlineStr">
+      <c r="K159" s="5" t="inlineStr"/>
+      <c r="L159" s="4" t="inlineStr"/>
+      <c r="M159" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -7452,7 +7920,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K160" s="4" t="inlineStr">
+      <c r="K160" s="5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L160" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M160" s="4" t="inlineStr">
         <is>
           <t>Chatbot-framed; 301 to voice pricing guide.</t>
         </is>
@@ -7499,7 +7977,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K161" s="4" t="inlineStr">
+      <c r="K161" s="5" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="L161" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M161" s="4" t="inlineStr">
         <is>
           <t>Merge tool into voice ROI model; 301.</t>
         </is>
@@ -7542,7 +8030,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K162" s="4" t="inlineStr">
+      <c r="K162" s="5" t="inlineStr"/>
+      <c r="L162" s="4" t="inlineStr"/>
+      <c r="M162" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -7585,7 +8075,9 @@
           <t>C · interlink/prune</t>
         </is>
       </c>
-      <c r="K163" s="4" t="inlineStr">
+      <c r="K163" s="5" t="inlineStr"/>
+      <c r="L163" s="4" t="inlineStr"/>
+      <c r="M163" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -7628,7 +8120,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K164" s="4" t="inlineStr">
+      <c r="K164" s="5" t="inlineStr"/>
+      <c r="L164" s="4" t="inlineStr"/>
+      <c r="M164" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -7671,7 +8165,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K165" s="4" t="inlineStr">
+      <c r="K165" s="5" t="inlineStr"/>
+      <c r="L165" s="4" t="inlineStr"/>
+      <c r="M165" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -7714,7 +8210,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K166" s="4" t="inlineStr">
+      <c r="K166" s="5" t="inlineStr"/>
+      <c r="L166" s="4" t="inlineStr"/>
+      <c r="M166" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -7757,7 +8255,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K167" s="4" t="inlineStr">
+      <c r="K167" s="5" t="inlineStr"/>
+      <c r="L167" s="4" t="inlineStr"/>
+      <c r="M167" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -7800,7 +8300,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K168" s="4" t="inlineStr">
+      <c r="K168" s="5" t="inlineStr"/>
+      <c r="L168" s="4" t="inlineStr"/>
+      <c r="M168" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -7843,7 +8345,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K169" s="4" t="inlineStr">
+      <c r="K169" s="5" t="inlineStr"/>
+      <c r="L169" s="4" t="inlineStr"/>
+      <c r="M169" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -7890,7 +8394,17 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K170" s="4" t="inlineStr">
+      <c r="K170" s="5" t="inlineStr">
+        <is>
+          <t>33.3</t>
+        </is>
+      </c>
+      <c r="L170" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM - review shared</t>
+        </is>
+      </c>
+      <c r="M170" s="4" t="inlineStr">
         <is>
           <t>Near-duplicate; merge + 301.</t>
         </is>
@@ -7933,7 +8447,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K171" s="4" t="inlineStr">
+      <c r="K171" s="5" t="inlineStr"/>
+      <c r="L171" s="4" t="inlineStr"/>
+      <c r="M171" s="4" t="inlineStr">
         <is>
           <t>Canonical profit-margins post.</t>
         </is>
@@ -7976,7 +8492,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K172" s="4" t="inlineStr">
+      <c r="K172" s="5" t="inlineStr"/>
+      <c r="L172" s="4" t="inlineStr"/>
+      <c r="M172" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -8019,7 +8537,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K173" s="4" t="inlineStr">
+      <c r="K173" s="5" t="inlineStr"/>
+      <c r="L173" s="4" t="inlineStr"/>
+      <c r="M173" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8062,7 +8582,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K174" s="4" t="inlineStr">
+      <c r="K174" s="5" t="inlineStr"/>
+      <c r="L174" s="4" t="inlineStr"/>
+      <c r="M174" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8105,7 +8627,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K175" s="4" t="inlineStr">
+      <c r="K175" s="5" t="inlineStr"/>
+      <c r="L175" s="4" t="inlineStr"/>
+      <c r="M175" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8148,7 +8672,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K176" s="4" t="inlineStr">
+      <c r="K176" s="5" t="inlineStr"/>
+      <c r="L176" s="4" t="inlineStr"/>
+      <c r="M176" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8191,7 +8717,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K177" s="4" t="inlineStr">
+      <c r="K177" s="5" t="inlineStr"/>
+      <c r="L177" s="4" t="inlineStr"/>
+      <c r="M177" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8234,7 +8762,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K178" s="4" t="inlineStr">
+      <c r="K178" s="5" t="inlineStr"/>
+      <c r="L178" s="4" t="inlineStr"/>
+      <c r="M178" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8281,7 +8811,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K179" s="4" t="inlineStr">
+      <c r="K179" s="5" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="L179" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M179" s="4" t="inlineStr">
         <is>
           <t>Off-topic (chatgpt); 301 to hub.</t>
         </is>
@@ -8324,7 +8864,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K180" s="4" t="inlineStr">
+      <c r="K180" s="5" t="inlineStr"/>
+      <c r="L180" s="4" t="inlineStr"/>
+      <c r="M180" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8367,7 +8909,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K181" s="4" t="inlineStr">
+      <c r="K181" s="5" t="inlineStr"/>
+      <c r="L181" s="4" t="inlineStr"/>
+      <c r="M181" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8410,7 +8954,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K182" s="4" t="inlineStr">
+      <c r="K182" s="5" t="inlineStr"/>
+      <c r="L182" s="4" t="inlineStr"/>
+      <c r="M182" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8453,7 +8999,9 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K183" s="4" t="inlineStr">
+      <c r="K183" s="5" t="inlineStr"/>
+      <c r="L183" s="4" t="inlineStr"/>
+      <c r="M183" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8500,9 +9048,19 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K184" s="4" t="inlineStr">
-        <is>
-          <t>Merge + 301.</t>
+      <c r="K184" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L184" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M184" s="4" t="inlineStr">
+        <is>
+          <t>Merge + 301. SURVIVOR REVIEW: this source has 13 queries vs 2 on the target — confirm which URL survives before 301.</t>
         </is>
       </c>
     </row>
@@ -8547,7 +9105,17 @@
           <t>A · deep revamp</t>
         </is>
       </c>
-      <c r="K185" s="4" t="inlineStr">
+      <c r="K185" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="L185" s="4" t="inlineStr">
+        <is>
+          <t>LOW - keep both</t>
+        </is>
+      </c>
+      <c r="M185" s="4" t="inlineStr">
         <is>
           <t>Chatbot build-vs-buy; 301 to canonical build-vs-buy.</t>
         </is>
@@ -8590,7 +9158,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K186" s="4" t="inlineStr">
+      <c r="K186" s="5" t="inlineStr"/>
+      <c r="L186" s="4" t="inlineStr"/>
+      <c r="M186" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8633,7 +9203,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K187" s="4" t="inlineStr">
+      <c r="K187" s="5" t="inlineStr"/>
+      <c r="L187" s="4" t="inlineStr"/>
+      <c r="M187" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -8676,7 +9248,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K188" s="4" t="inlineStr">
+      <c r="K188" s="5" t="inlineStr"/>
+      <c r="L188" s="4" t="inlineStr"/>
+      <c r="M188" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -8719,7 +9293,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K189" s="4" t="inlineStr">
+      <c r="K189" s="5" t="inlineStr"/>
+      <c r="L189" s="4" t="inlineStr"/>
+      <c r="M189" s="4" t="inlineStr">
         <is>
           <t>Revamp under the program hub.</t>
         </is>
@@ -8762,7 +9338,9 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K190" s="4" t="inlineStr">
+      <c r="K190" s="5" t="inlineStr"/>
+      <c r="L190" s="4" t="inlineStr"/>
+      <c r="M190" s="4" t="inlineStr">
         <is>
           <t>Revamp; link from voice-ai-agency-referral-program.</t>
         </is>
@@ -8805,14 +9383,16 @@
           <t>B · light revamp</t>
         </is>
       </c>
-      <c r="K191" s="4" t="inlineStr">
+      <c r="K191" s="5" t="inlineStr"/>
+      <c r="L191" s="4" t="inlineStr"/>
+      <c r="M191" s="4" t="inlineStr">
         <is>
           <t>Revamp under the program hub; wire Academy posts to it.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K191"/>
+  <autoFilter ref="A1:M191"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8859,7 +9439,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -8879,7 +9459,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6">
@@ -8899,7 +9479,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -8909,7 +9489,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Vet plan with Tier-1 GSC pulls: /agency duplicate + receptionist winner
Page-query and money-term data surfaced two corrections:
- /agency is a byte-identical duplicate of /whitelabel (canonical ignored,
  not in sitemap) ranking separately for head terms -> add 301 to /whitelabel.
- best-white-label-ai-receptionist ranks pos 6.5 / 17 clicks for "white
  label ai receptionist" (top non-brand converter) -> reverse its merge,
  make it canonical for the receptionist money term.
Also confirms severe head-term cannibalisation across 8-13 URLs and the
chatbot pages' unconvertible impressions. Raw pulls archived.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UhVChLeNNjFDr6eASTMGhh
</commit_message>
<xml_diff>
--- a/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
+++ b/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Data findings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Redirect map'!$A$1:$M$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Redirect map'!$A$1:$M$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M191"/>
+  <dimension ref="A1:M192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2406,16 +2406,12 @@
           <t>2 · Agency Academy</t>
         </is>
       </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>/blogs/top-10-white-label-voice-ai-platforms-for-agencies-2026</t>
-        </is>
-      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>CANONICAL</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="5" t="n">
         <v>12333</v>
       </c>
@@ -2445,7 +2441,7 @@
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>Fold into canonical roundup; 301.</t>
+          <t>GSC: pos 6.5 for "white label ai receptionist", 17 clicks (top non-brand converter in the cluster). Keep as canonical for the receptionist money term - do NOT merge.</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5147,7 @@
       <c r="L99" s="4" t="inlineStr"/>
       <c r="M99" s="4" t="inlineStr">
         <is>
-          <t>Canonical "best white-label voice AI" roundup. Rewrite as honest named comparison + current data.</t>
+          <t>Canonical "best white-label voice AI PLATFORMS" roundup (platforms intent). GSC: 130-533 impr on head terms but pos 19-25. best-white-label-ai-receptionist is a SEPARATE winner (receptionist intent) and is NOT merged in.</t>
         </is>
       </c>
     </row>
@@ -9391,8 +9387,57 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>/agency</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>2 · Agency Academy</t>
+        </is>
+      </c>
+      <c r="D192" s="12" t="inlineStr">
+        <is>
+          <t>REDIRECT</t>
+        </is>
+      </c>
+      <c r="E192" s="4" t="inlineStr">
+        <is>
+          <t>/whitelabel</t>
+        </is>
+      </c>
+      <c r="F192" s="5" t="n">
+        <v>10419</v>
+      </c>
+      <c r="G192" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="H192" s="5" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="I192" s="5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J192" s="6" t="inlineStr">
+        <is>
+          <t>A · deep revamp</t>
+        </is>
+      </c>
+      <c r="K192" s="5" t="inlineStr"/>
+      <c r="L192" s="4" t="inlineStr"/>
+      <c r="M192" s="4" t="inlineStr">
+        <is>
+          <t>DUPLICATE of /whitelabel (byte-identical, canonical already points to /whitelabel but is being IGNORED). Not in sitemap yet ranks separately/above /whitelabel for head terms (e.g. pos 39 for "white label ai voice agent", 284 impr). 301 /agency to /whitelabel and remove internal links. GSC-confirmed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M191"/>
+  <autoFilter ref="A1:M192"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9439,7 +9484,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -9469,7 +9514,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -9479,7 +9524,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -9531,7 +9576,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -9593,7 +9638,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Correct /agency: already 308-redirected to /whitelabel (no action)
Verified with a no-follow request: /agency returns HTTP 308 -> /whitelabel
(permanent). Earlier -L fetch followed it and misread identical bytes as a
duplicate. Mark it DONE, not an action item; its historical head-term
impressions will consolidate into /whitelabel like the apex/www fix. Only
residual check: ensure no internal links still point to /agency.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UhVChLeNNjFDr6eASTMGhh
</commit_message>
<xml_diff>
--- a/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
+++ b/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
@@ -49,7 +49,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -106,6 +106,11 @@
         <fgColor rgb="00CFE0FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9F0DC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -133,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -178,6 +183,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -9401,9 +9409,9 @@
           <t>2 · Agency Academy</t>
         </is>
       </c>
-      <c r="D192" s="12" t="inlineStr">
-        <is>
-          <t>REDIRECT</t>
+      <c r="D192" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
@@ -9432,7 +9440,7 @@
       <c r="L192" s="4" t="inlineStr"/>
       <c r="M192" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE of /whitelabel (byte-identical, canonical already points to /whitelabel but is being IGNORED). Not in sitemap yet ranks separately/above /whitelabel for head terms (e.g. pos 39 for "white label ai voice agent", 284 impr). 301 /agency to /whitelabel and remove internal links. GSC-confirmed.</t>
+          <t>ALREADY 308-redirected to /whitelabel (permanent; passes signal like a 301) - NO ACTION. Its historical head-term impressions in the 16-mo data will consolidate into /whitelabel as Google reprocesses (same as the apex/www fix). Only verify no internal links still point to /agency.</t>
         </is>
       </c>
     </row>
@@ -9456,19 +9464,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
@@ -9478,7 +9486,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>CANONICAL</t>
         </is>
@@ -9488,7 +9496,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>REVAMP</t>
         </is>
@@ -9498,7 +9506,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
@@ -9508,7 +9516,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>MERGE</t>
         </is>
@@ -9518,17 +9526,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>REDIRECT</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>REFRAME</t>
         </is>
@@ -9538,12 +9546,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Pillar</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
@@ -9620,12 +9628,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Revamp tier (GSC-grounded)</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
@@ -9700,144 +9708,144 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Finding</t>
         </is>
       </c>
-      <c r="B1" s="24" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Window</t>
         </is>
       </c>
-      <c r="B2" s="26" t="inlineStr">
+      <c r="B2" s="27" t="inlineStr">
         <is>
           <t>16 months (2025-05-07 to 2026-09-06), Web search</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Site total</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>18,848 clicks · 1,908,737 impressions · 0.99% CTR</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Trend</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>Impressions grew ~46x as programmatic content shipped (13.5k -&gt; 621k per 90 days); clicks only ~1.8x; CTR fell 19.85% -&gt; 0.76%. Relevance/snippet failure at scale, confirmed — this (not host duplication) is now the primary problem.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Apex/www — RESOLVED</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>Host duplication has been canonicalised to a single host (no longer a lever). The 16-mo export still shows both hosts historically; tiers here are deduped by path, i.e. the consolidated single-URL view. Re-pull GSC in 4-8 weeks to measure the consolidation lift.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>WL cluster</t>
         </is>
       </c>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="27" t="inlineStr">
         <is>
           <t>764,907 impressions = 40% of all site impressions, but only 2,036 clicks @ 0.27% CTR (vs 0.99% site).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Revamp prize (#1 lever now)</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>93 WL pages sit in striking distance (pos&lt;=20, impr&gt;=1000, CTR&lt;1.5%) holding ~721,000 impressions — the Tier-A revamp target and, with apex/www done, the single biggest lever. Note: exclude chatbot-query impressions (structurally unconvertible for a voice product) from any CTR-lift forecast.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Chatbot = wasted impressions</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>'white label chatbot' 1,569 impr pos 18.9 0.13%; 'chatbot white label' 1,354; 'white label ai chatbot' 1,003; 'whitelabel chatbot' 939; all ~0% CTR. Voice-first Trillet can't convert chatbot demand — reframe/redirect confirmed.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Voice/receptionist converts</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>'white label ai receptionist' 1,549 impr, 37 clk, 2.39% CTR (best non-brand); 'ai receptionist white label' 1.59%; 'retell ai white label' 3.35%. 10-20x better than chatbot terms at similar positions.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Head terms stuck</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>'white label ai voice agent' pos 26.8; 'white label ai platform' pos 30.6; 'white label voice' pos 19.7 — the terms the /whitelabel hub must win are on page 2-3 today.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>Brand WL demand</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>'trillet white label' 46.73% CTR; 'trillet ai white label' 21.70%. Real branded white-label demand exists and converts.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Worst offenders (page)</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>voice-ai-white-label-pricing-breakdown-2026 42,150 impr @0.06%; best-white-label-ai-chatbot 39,390 @0.19%; voicify-alternative 26,793 impr @0.00% (1 click).</t>
         </is>

</xml_diff>

<commit_message>
Vet every map URL against live HTTP; add Live HTTP column
Checked all 190 source URLs no-follow. Result: 184 live 200s, 6 "404 (to
build)" = the planned NEW pages, 1 already-308 (/agency, DONE). No hidden
redirects or already-gone pages among the merge/redirect/keep sources, so
no planned action is redundant. Live HTTP recorded as a column; raw status
archived.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UhVChLeNNjFDr6eASTMGhh
</commit_message>
<xml_diff>
--- a/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
+++ b/seo-audit/Trillet-WhiteLabel-Redirect-Map.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Data findings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Redirect map'!$A$1:$M$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Redirect map'!$A$1:$N$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M192"/>
+  <dimension ref="A1:N192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -583,7 +583,8 @@
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="58" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="58" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -649,6 +650,11 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Live HTTP</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Reason / note</t>
         </is>
       </c>
@@ -692,7 +698,12 @@
       </c>
       <c r="K2" s="5" t="inlineStr"/>
       <c r="L2" s="4" t="inlineStr"/>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>Rebuild as the cluster hub (title/H1/subhead, SoftwareApplication+Offer schema, remove meta-kw, links to all spokes).</t>
         </is>
@@ -737,7 +748,12 @@
       </c>
       <c r="K3" s="5" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr"/>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Canonical pricing target. Point all WL-pricing blogs here.</t>
         </is>
@@ -782,7 +798,12 @@
       </c>
       <c r="K4" s="5" t="inlineStr"/>
       <c r="L4" s="4" t="inlineStr"/>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Rebuild as partner-program hub (Reseller/OEM/Referral/Agency tiers, benefits, apply CTA).</t>
         </is>
@@ -819,7 +840,12 @@
       </c>
       <c r="K5" s="5" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>404 (to build)</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>NEW integrations directory hub.</t>
         </is>
@@ -856,7 +882,12 @@
       </c>
       <c r="K6" s="5" t="inlineStr"/>
       <c r="L6" s="4" t="inlineStr"/>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>404 (to build)</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>NEW canonical GoHighLevel landing page (consolidates GHL posts as spokes).</t>
         </is>
@@ -893,7 +924,12 @@
       </c>
       <c r="K7" s="5" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr"/>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>404 (to build)</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>NEW AI Voice Agency Academy hub — organises the ~45 business posts into a learning path.</t>
         </is>
@@ -930,7 +966,12 @@
       </c>
       <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="4" t="inlineStr"/>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>404 (to build)</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>NEW white-label-by-industry index — links the ~25 vertical posts + their /receptionist/industries counterparts.</t>
         </is>
@@ -967,7 +1008,12 @@
       </c>
       <c r="K9" s="5" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr"/>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>404 (to build)</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>NEW compare &amp; alternatives index — links all vs/alternative pages, one per competitor.</t>
         </is>
@@ -1004,7 +1050,12 @@
       </c>
       <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr"/>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>404 (to build)</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>NEW /reviews social-proof hub (Review schema).</t>
         </is>
@@ -1049,7 +1100,12 @@
       </c>
       <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1094,7 +1150,12 @@
       </c>
       <c r="K12" s="5" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1139,7 +1200,12 @@
       </c>
       <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Distinct 60-day-plan format (only 2 queries). Pair with the reframed how-to-start page; consider merging later.</t>
         </is>
@@ -1184,7 +1250,12 @@
       </c>
       <c r="K14" s="5" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -1229,7 +1300,12 @@
       </c>
       <c r="K15" s="5" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1274,7 +1350,12 @@
       </c>
       <c r="K16" s="5" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1319,7 +1400,12 @@
       </c>
       <c r="K17" s="5" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1364,7 +1450,12 @@
       </c>
       <c r="K18" s="5" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1409,7 +1500,12 @@
       </c>
       <c r="K19" s="5" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr"/>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1454,7 +1550,12 @@
       </c>
       <c r="K20" s="5" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1511,7 +1612,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>Chatbot; 301 to voice canvas.</t>
         </is>
@@ -1556,7 +1662,12 @@
       </c>
       <c r="K22" s="5" t="inlineStr"/>
       <c r="L22" s="4" t="inlineStr"/>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1601,7 +1712,12 @@
       </c>
       <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr"/>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1646,7 +1762,12 @@
       </c>
       <c r="K24" s="5" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr"/>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1691,7 +1812,12 @@
       </c>
       <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="4" t="inlineStr"/>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -1736,7 +1862,12 @@
       </c>
       <c r="K26" s="5" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -1781,7 +1912,12 @@
       </c>
       <c r="K27" s="5" t="inlineStr"/>
       <c r="L27" s="4" t="inlineStr"/>
-      <c r="M27" s="4" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -1826,7 +1962,12 @@
       </c>
       <c r="K28" s="5" t="inlineStr"/>
       <c r="L28" s="4" t="inlineStr"/>
-      <c r="M28" s="4" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -1871,7 +2012,12 @@
       </c>
       <c r="K29" s="5" t="inlineStr"/>
       <c r="L29" s="4" t="inlineStr"/>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1916,7 +2062,12 @@
       </c>
       <c r="K30" s="5" t="inlineStr"/>
       <c r="L30" s="4" t="inlineStr"/>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -1961,7 +2112,12 @@
       </c>
       <c r="K31" s="5" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr"/>
-      <c r="M31" s="4" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2018,7 +2174,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M32" s="4" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
         <is>
           <t>Fold into the canonical pricing guide; 301.</t>
         </is>
@@ -2063,7 +2224,12 @@
       </c>
       <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="4" t="inlineStr"/>
-      <c r="M33" s="4" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>Canonical agency-economics post.</t>
         </is>
@@ -2108,7 +2274,12 @@
       </c>
       <c r="K34" s="5" t="inlineStr"/>
       <c r="L34" s="4" t="inlineStr"/>
-      <c r="M34" s="4" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2145,7 +2316,12 @@
       </c>
       <c r="K35" s="5" t="inlineStr"/>
       <c r="L35" s="4" t="inlineStr"/>
-      <c r="M35" s="4" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2190,7 +2366,12 @@
       </c>
       <c r="K36" s="5" t="inlineStr"/>
       <c r="L36" s="4" t="inlineStr"/>
-      <c r="M36" s="4" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2235,7 +2416,12 @@
       </c>
       <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr"/>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2280,7 +2466,12 @@
       </c>
       <c r="K38" s="5" t="inlineStr"/>
       <c r="L38" s="4" t="inlineStr"/>
-      <c r="M38" s="4" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -2337,7 +2528,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M39" s="4" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
         <is>
           <t>Fold into canonical roundup; 301.</t>
         </is>
@@ -2394,7 +2590,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M40" s="4" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
         <is>
           <t>Chatbot-framed; 301 to voice roundup.</t>
         </is>
@@ -2447,7 +2648,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M41" s="4" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
         <is>
           <t>GSC: pos 6.5 for "white label ai receptionist", 17 clicks (top non-brand converter in the cluster). Keep as canonical for the receptionist money term - do NOT merge.</t>
         </is>
@@ -2492,7 +2698,12 @@
       </c>
       <c r="K42" s="5" t="inlineStr"/>
       <c r="L42" s="4" t="inlineStr"/>
-      <c r="M42" s="4" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
         <is>
           <t>Distinct build-vs-buy angle; keep as canonical build-vs-buy.</t>
         </is>
@@ -2537,7 +2748,12 @@
       </c>
       <c r="K43" s="5" t="inlineStr"/>
       <c r="L43" s="4" t="inlineStr"/>
-      <c r="M43" s="4" t="inlineStr">
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2582,7 +2798,12 @@
       </c>
       <c r="K44" s="5" t="inlineStr"/>
       <c r="L44" s="4" t="inlineStr"/>
-      <c r="M44" s="4" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2627,7 +2848,12 @@
       </c>
       <c r="K45" s="5" t="inlineStr"/>
       <c r="L45" s="4" t="inlineStr"/>
-      <c r="M45" s="4" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2672,7 +2898,12 @@
       </c>
       <c r="K46" s="5" t="inlineStr"/>
       <c r="L46" s="4" t="inlineStr"/>
-      <c r="M46" s="4" t="inlineStr">
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N46" s="4" t="inlineStr">
         <is>
           <t>Distinct "cheapest" price intent; keep, link to hub + pricing guide.</t>
         </is>
@@ -2717,7 +2948,12 @@
       </c>
       <c r="K47" s="5" t="inlineStr"/>
       <c r="L47" s="4" t="inlineStr"/>
-      <c r="M47" s="4" t="inlineStr">
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2762,7 +2998,12 @@
       </c>
       <c r="K48" s="5" t="inlineStr"/>
       <c r="L48" s="4" t="inlineStr"/>
-      <c r="M48" s="4" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N48" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2807,7 +3048,12 @@
       </c>
       <c r="K49" s="5" t="inlineStr"/>
       <c r="L49" s="4" t="inlineStr"/>
-      <c r="M49" s="4" t="inlineStr">
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2852,7 +3098,12 @@
       </c>
       <c r="K50" s="5" t="inlineStr"/>
       <c r="L50" s="4" t="inlineStr"/>
-      <c r="M50" s="4" t="inlineStr">
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N50" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2897,7 +3148,12 @@
       </c>
       <c r="K51" s="5" t="inlineStr"/>
       <c r="L51" s="4" t="inlineStr"/>
-      <c r="M51" s="4" t="inlineStr">
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -2942,7 +3198,12 @@
       </c>
       <c r="K52" s="5" t="inlineStr"/>
       <c r="L52" s="4" t="inlineStr"/>
-      <c r="M52" s="4" t="inlineStr">
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N52" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -2999,7 +3260,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M53" s="4" t="inlineStr">
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N53" s="4" t="inlineStr">
         <is>
           <t>Fold into canonical roundup; 301.</t>
         </is>
@@ -3044,7 +3310,12 @@
       </c>
       <c r="K54" s="5" t="inlineStr"/>
       <c r="L54" s="4" t="inlineStr"/>
-      <c r="M54" s="4" t="inlineStr">
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3089,7 +3360,12 @@
       </c>
       <c r="K55" s="5" t="inlineStr"/>
       <c r="L55" s="4" t="inlineStr"/>
-      <c r="M55" s="4" t="inlineStr">
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3134,7 +3410,12 @@
       </c>
       <c r="K56" s="5" t="inlineStr"/>
       <c r="L56" s="4" t="inlineStr"/>
-      <c r="M56" s="4" t="inlineStr">
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
         <is>
           <t>Distinct how-to; keep as GHL spoke.</t>
         </is>
@@ -3191,7 +3472,12 @@
           <t>MEDIUM - review shared</t>
         </is>
       </c>
-      <c r="M57" s="4" t="inlineStr">
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
         <is>
           <t>Same intent; merge + 301.</t>
         </is>
@@ -3236,7 +3522,12 @@
       </c>
       <c r="K58" s="5" t="inlineStr"/>
       <c r="L58" s="4" t="inlineStr"/>
-      <c r="M58" s="4" t="inlineStr">
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
         <is>
           <t>Distinct angle; keep as GHL spoke.</t>
         </is>
@@ -3293,7 +3584,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M59" s="4" t="inlineStr">
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
         <is>
           <t>Fold into the new GHL landing page; 301.</t>
         </is>
@@ -3350,7 +3646,12 @@
           <t>MEDIUM - review shared</t>
         </is>
       </c>
-      <c r="M60" s="4" t="inlineStr">
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
         <is>
           <t>Same intent; merge + 301.</t>
         </is>
@@ -3395,7 +3696,12 @@
       </c>
       <c r="K61" s="5" t="inlineStr"/>
       <c r="L61" s="4" t="inlineStr"/>
-      <c r="M61" s="4" t="inlineStr">
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -3440,7 +3746,12 @@
       </c>
       <c r="K62" s="5" t="inlineStr"/>
       <c r="L62" s="4" t="inlineStr"/>
-      <c r="M62" s="4" t="inlineStr">
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3489,7 +3800,12 @@
           <t>SOURCE HAS NO QUERIES - safe to redirect</t>
         </is>
       </c>
-      <c r="M63" s="4" t="inlineStr">
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
         <is>
           <t>Chatbot definitional; 301 to voice.</t>
         </is>
@@ -3534,7 +3850,12 @@
       </c>
       <c r="K64" s="5" t="inlineStr"/>
       <c r="L64" s="4" t="inlineStr"/>
-      <c r="M64" s="4" t="inlineStr">
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N64" s="4" t="inlineStr">
         <is>
           <t>Distinct cost-to-start intent; keep.</t>
         </is>
@@ -3591,7 +3912,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M65" s="4" t="inlineStr">
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N65" s="4" t="inlineStr">
         <is>
           <t>Same intent; merge + 301.</t>
         </is>
@@ -3636,7 +3962,12 @@
       </c>
       <c r="K66" s="5" t="inlineStr"/>
       <c r="L66" s="4" t="inlineStr"/>
-      <c r="M66" s="4" t="inlineStr">
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N66" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3681,7 +4012,12 @@
       </c>
       <c r="K67" s="5" t="inlineStr"/>
       <c r="L67" s="4" t="inlineStr"/>
-      <c r="M67" s="4" t="inlineStr">
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3738,7 +4074,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M68" s="4" t="inlineStr">
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N68" s="4" t="inlineStr">
         <is>
           <t>Chatbot; 301 to voice features checklist.</t>
         </is>
@@ -3783,7 +4124,12 @@
       </c>
       <c r="K69" s="5" t="inlineStr"/>
       <c r="L69" s="4" t="inlineStr"/>
-      <c r="M69" s="4" t="inlineStr">
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3828,7 +4174,12 @@
       </c>
       <c r="K70" s="5" t="inlineStr"/>
       <c r="L70" s="4" t="inlineStr"/>
-      <c r="M70" s="4" t="inlineStr">
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N70" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3873,7 +4224,12 @@
       </c>
       <c r="K71" s="5" t="inlineStr"/>
       <c r="L71" s="4" t="inlineStr"/>
-      <c r="M71" s="4" t="inlineStr">
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N71" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -3926,7 +4282,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M72" s="4" t="inlineStr">
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N72" s="4" t="inlineStr">
         <is>
           <t>GSC: 96 queries — too much traffic to redirect. Rewrite to voice framing ("how to start a voice AI agency") and keep the URL as a primary start guide.</t>
         </is>
@@ -3971,7 +4332,12 @@
       </c>
       <c r="K73" s="5" t="inlineStr"/>
       <c r="L73" s="4" t="inlineStr"/>
-      <c r="M73" s="4" t="inlineStr">
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -4016,7 +4382,12 @@
       </c>
       <c r="K74" s="5" t="inlineStr"/>
       <c r="L74" s="4" t="inlineStr"/>
-      <c r="M74" s="4" t="inlineStr">
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N74" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4061,7 +4432,12 @@
       </c>
       <c r="K75" s="5" t="inlineStr"/>
       <c r="L75" s="4" t="inlineStr"/>
-      <c r="M75" s="4" t="inlineStr">
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N75" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -4106,7 +4482,12 @@
       </c>
       <c r="K76" s="5" t="inlineStr"/>
       <c r="L76" s="4" t="inlineStr"/>
-      <c r="M76" s="4" t="inlineStr">
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N76" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4151,7 +4532,12 @@
       </c>
       <c r="K77" s="5" t="inlineStr"/>
       <c r="L77" s="4" t="inlineStr"/>
-      <c r="M77" s="4" t="inlineStr">
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N77" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -4196,7 +4582,12 @@
       </c>
       <c r="K78" s="5" t="inlineStr"/>
       <c r="L78" s="4" t="inlineStr"/>
-      <c r="M78" s="4" t="inlineStr">
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N78" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -4241,7 +4632,12 @@
       </c>
       <c r="K79" s="5" t="inlineStr"/>
       <c r="L79" s="4" t="inlineStr"/>
-      <c r="M79" s="4" t="inlineStr">
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N79" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -4286,7 +4682,12 @@
       </c>
       <c r="K80" s="5" t="inlineStr"/>
       <c r="L80" s="4" t="inlineStr"/>
-      <c r="M80" s="4" t="inlineStr">
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N80" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4331,7 +4732,12 @@
       </c>
       <c r="K81" s="5" t="inlineStr"/>
       <c r="L81" s="4" t="inlineStr"/>
-      <c r="M81" s="4" t="inlineStr">
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N81" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4388,7 +4794,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M82" s="4" t="inlineStr">
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N82" s="4" t="inlineStr">
         <is>
           <t>Same intent; merge as a section + 301.</t>
         </is>
@@ -4433,7 +4844,12 @@
       </c>
       <c r="K83" s="5" t="inlineStr"/>
       <c r="L83" s="4" t="inlineStr"/>
-      <c r="M83" s="4" t="inlineStr">
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N83" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -4478,7 +4894,12 @@
       </c>
       <c r="K84" s="5" t="inlineStr"/>
       <c r="L84" s="4" t="inlineStr"/>
-      <c r="M84" s="4" t="inlineStr">
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N84" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): ranks #2 for "my ai front desk alternative" — distinct intent from the vs.</t>
         </is>
@@ -4523,7 +4944,12 @@
       </c>
       <c r="K85" s="5" t="inlineStr"/>
       <c r="L85" s="4" t="inlineStr"/>
-      <c r="M85" s="4" t="inlineStr">
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N85" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): distinct white-label angle; differentiate from alternative-2026 (general) and the vs (head-to-head).</t>
         </is>
@@ -4568,7 +4994,12 @@
       </c>
       <c r="K86" s="5" t="inlineStr"/>
       <c r="L86" s="4" t="inlineStr"/>
-      <c r="M86" s="4" t="inlineStr">
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N86" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -4613,7 +5044,12 @@
       </c>
       <c r="K87" s="5" t="inlineStr"/>
       <c r="L87" s="4" t="inlineStr"/>
-      <c r="M87" s="4" t="inlineStr">
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N87" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -4658,7 +5094,12 @@
       </c>
       <c r="K88" s="5" t="inlineStr"/>
       <c r="L88" s="4" t="inlineStr"/>
-      <c r="M88" s="4" t="inlineStr">
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N88" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4703,7 +5144,12 @@
       </c>
       <c r="K89" s="5" t="inlineStr"/>
       <c r="L89" s="4" t="inlineStr"/>
-      <c r="M89" s="4" t="inlineStr">
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N89" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4748,7 +5194,12 @@
       </c>
       <c r="K90" s="5" t="inlineStr"/>
       <c r="L90" s="4" t="inlineStr"/>
-      <c r="M90" s="4" t="inlineStr">
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N90" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4793,7 +5244,12 @@
       </c>
       <c r="K91" s="5" t="inlineStr"/>
       <c r="L91" s="4" t="inlineStr"/>
-      <c r="M91" s="4" t="inlineStr">
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N91" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -4838,7 +5294,12 @@
       </c>
       <c r="K92" s="5" t="inlineStr"/>
       <c r="L92" s="4" t="inlineStr"/>
-      <c r="M92" s="4" t="inlineStr">
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N92" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): owns the converting "retell ai white label" niche (3.35% CTR); distinct intent from the head-to-head vs.</t>
         </is>
@@ -4883,7 +5344,12 @@
       </c>
       <c r="K93" s="5" t="inlineStr"/>
       <c r="L93" s="4" t="inlineStr"/>
-      <c r="M93" s="4" t="inlineStr">
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N93" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): "smith ai alternative" is roundup intent, distinct from the head-to-head vs.</t>
         </is>
@@ -4928,7 +5394,12 @@
       </c>
       <c r="K94" s="5" t="inlineStr"/>
       <c r="L94" s="4" t="inlineStr"/>
-      <c r="M94" s="4" t="inlineStr">
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N94" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -4973,7 +5444,12 @@
       </c>
       <c r="K95" s="5" t="inlineStr"/>
       <c r="L95" s="4" t="inlineStr"/>
-      <c r="M95" s="4" t="inlineStr">
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N95" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): distinct agency-angle content; co-ranks only on the brand term. Differentiate from the vs.</t>
         </is>
@@ -5018,7 +5494,12 @@
       </c>
       <c r="K96" s="5" t="inlineStr"/>
       <c r="L96" s="4" t="inlineStr"/>
-      <c r="M96" s="4" t="inlineStr">
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N96" s="4" t="inlineStr">
         <is>
           <t>Canonical head-to-head. synthflow-alternative-for-agencies has distinct content and is KEPT (SERP-validated).</t>
         </is>
@@ -5063,7 +5544,12 @@
       </c>
       <c r="K97" s="5" t="inlineStr"/>
       <c r="L97" s="4" t="inlineStr"/>
-      <c r="M97" s="4" t="inlineStr">
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N97" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5108,7 +5594,12 @@
       </c>
       <c r="K98" s="5" t="inlineStr"/>
       <c r="L98" s="4" t="inlineStr"/>
-      <c r="M98" s="4" t="inlineStr">
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N98" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5153,7 +5644,12 @@
       </c>
       <c r="K99" s="5" t="inlineStr"/>
       <c r="L99" s="4" t="inlineStr"/>
-      <c r="M99" s="4" t="inlineStr">
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N99" s="4" t="inlineStr">
         <is>
           <t>Canonical "best white-label voice AI PLATFORMS" roundup (platforms intent). GSC: 130-533 impr on head terms but pos 19-25. best-white-label-ai-receptionist is a SEPARATE winner (receptionist intent) and is NOT merged in.</t>
         </is>
@@ -5198,7 +5694,12 @@
       </c>
       <c r="K100" s="5" t="inlineStr"/>
       <c r="L100" s="4" t="inlineStr"/>
-      <c r="M100" s="4" t="inlineStr">
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N100" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5243,7 +5744,12 @@
       </c>
       <c r="K101" s="5" t="inlineStr"/>
       <c r="L101" s="4" t="inlineStr"/>
-      <c r="M101" s="4" t="inlineStr">
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N101" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5288,7 +5794,12 @@
       </c>
       <c r="K102" s="5" t="inlineStr"/>
       <c r="L102" s="4" t="inlineStr"/>
-      <c r="M102" s="4" t="inlineStr">
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N102" s="4" t="inlineStr">
         <is>
           <t>Canonical "GHL native vs Trillet" comparison.</t>
         </is>
@@ -5333,7 +5844,12 @@
       </c>
       <c r="K103" s="5" t="inlineStr"/>
       <c r="L103" s="4" t="inlineStr"/>
-      <c r="M103" s="4" t="inlineStr">
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N103" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5378,7 +5894,12 @@
       </c>
       <c r="K104" s="5" t="inlineStr"/>
       <c r="L104" s="4" t="inlineStr"/>
-      <c r="M104" s="4" t="inlineStr">
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N104" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5423,7 +5944,12 @@
       </c>
       <c r="K105" s="5" t="inlineStr"/>
       <c r="L105" s="4" t="inlineStr"/>
-      <c r="M105" s="4" t="inlineStr">
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N105" s="4" t="inlineStr">
         <is>
           <t>Canonical head-to-head. The two MAFD alternative pages serve different intent and are KEPT (SERP-validated), not merged here.</t>
         </is>
@@ -5468,7 +5994,12 @@
       </c>
       <c r="K106" s="5" t="inlineStr"/>
       <c r="L106" s="4" t="inlineStr"/>
-      <c r="M106" s="4" t="inlineStr">
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N106" s="4" t="inlineStr">
         <is>
           <t>Canonical head-to-head. The Retell/Vapi white-label "alternative" pages own distinct intent and are KEPT (SERP-validated).</t>
         </is>
@@ -5513,7 +6044,12 @@
       </c>
       <c r="K107" s="5" t="inlineStr"/>
       <c r="L107" s="4" t="inlineStr"/>
-      <c r="M107" s="4" t="inlineStr">
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N107" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5558,7 +6094,12 @@
       </c>
       <c r="K108" s="5" t="inlineStr"/>
       <c r="L108" s="4" t="inlineStr"/>
-      <c r="M108" s="4" t="inlineStr">
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N108" s="4" t="inlineStr">
         <is>
           <t>Canonical head-to-head. smith-ai-alternative-2026 owns roundup intent and is KEPT (SERP-validated).</t>
         </is>
@@ -5603,7 +6144,12 @@
       </c>
       <c r="K109" s="5" t="inlineStr"/>
       <c r="L109" s="4" t="inlineStr"/>
-      <c r="M109" s="4" t="inlineStr">
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N109" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5648,7 +6194,12 @@
       </c>
       <c r="K110" s="5" t="inlineStr"/>
       <c r="L110" s="4" t="inlineStr"/>
-      <c r="M110" s="4" t="inlineStr">
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N110" s="4" t="inlineStr">
         <is>
           <t>SERP-validated (keep): ranks p1 (#3) for "vapi alternative for agencies" — roundup intent, distinct from the vs.</t>
         </is>
@@ -5693,7 +6244,12 @@
       </c>
       <c r="K111" s="5" t="inlineStr"/>
       <c r="L111" s="4" t="inlineStr"/>
-      <c r="M111" s="4" t="inlineStr">
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N111" s="4" t="inlineStr">
         <is>
           <t>Distinct compliance angle (the wedge); keep.</t>
         </is>
@@ -5738,7 +6294,12 @@
       </c>
       <c r="K112" s="5" t="inlineStr"/>
       <c r="L112" s="4" t="inlineStr"/>
-      <c r="M112" s="4" t="inlineStr">
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N112" s="4" t="inlineStr">
         <is>
           <t>Distinct: Vapi own WL options; keep.</t>
         </is>
@@ -5783,7 +6344,12 @@
       </c>
       <c r="K113" s="5" t="inlineStr"/>
       <c r="L113" s="4" t="inlineStr"/>
-      <c r="M113" s="4" t="inlineStr">
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N113" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -5828,7 +6394,12 @@
       </c>
       <c r="K114" s="5" t="inlineStr"/>
       <c r="L114" s="4" t="inlineStr"/>
-      <c r="M114" s="4" t="inlineStr">
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N114" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -5873,7 +6444,12 @@
       </c>
       <c r="K115" s="5" t="inlineStr"/>
       <c r="L115" s="4" t="inlineStr"/>
-      <c r="M115" s="4" t="inlineStr">
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N115" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -5918,7 +6494,12 @@
       </c>
       <c r="K116" s="5" t="inlineStr"/>
       <c r="L116" s="4" t="inlineStr"/>
-      <c r="M116" s="4" t="inlineStr">
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N116" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -5963,7 +6544,12 @@
       </c>
       <c r="K117" s="5" t="inlineStr"/>
       <c r="L117" s="4" t="inlineStr"/>
-      <c r="M117" s="4" t="inlineStr">
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N117" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6008,7 +6594,12 @@
       </c>
       <c r="K118" s="5" t="inlineStr"/>
       <c r="L118" s="4" t="inlineStr"/>
-      <c r="M118" s="4" t="inlineStr">
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N118" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6053,7 +6644,12 @@
       </c>
       <c r="K119" s="5" t="inlineStr"/>
       <c r="L119" s="4" t="inlineStr"/>
-      <c r="M119" s="4" t="inlineStr">
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N119" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6098,7 +6694,12 @@
       </c>
       <c r="K120" s="5" t="inlineStr"/>
       <c r="L120" s="4" t="inlineStr"/>
-      <c r="M120" s="4" t="inlineStr">
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N120" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -6135,7 +6736,12 @@
       </c>
       <c r="K121" s="5" t="inlineStr"/>
       <c r="L121" s="4" t="inlineStr"/>
-      <c r="M121" s="4" t="inlineStr">
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N121" s="4" t="inlineStr">
         <is>
           <t>KEEP but sharpen "sell voice, not chat"; the chatbot-&gt;voice converter.</t>
         </is>
@@ -6180,7 +6786,12 @@
       </c>
       <c r="K122" s="5" t="inlineStr"/>
       <c r="L122" s="4" t="inlineStr"/>
-      <c r="M122" s="4" t="inlineStr">
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N122" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -6225,7 +6836,12 @@
       </c>
       <c r="K123" s="5" t="inlineStr"/>
       <c r="L123" s="4" t="inlineStr"/>
-      <c r="M123" s="4" t="inlineStr">
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N123" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -6270,7 +6886,12 @@
       </c>
       <c r="K124" s="5" t="inlineStr"/>
       <c r="L124" s="4" t="inlineStr"/>
-      <c r="M124" s="4" t="inlineStr">
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N124" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -6315,7 +6936,12 @@
       </c>
       <c r="K125" s="5" t="inlineStr"/>
       <c r="L125" s="4" t="inlineStr"/>
-      <c r="M125" s="4" t="inlineStr">
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N125" s="4" t="inlineStr">
         <is>
           <t>Distinct ROI tool; keep.</t>
         </is>
@@ -6364,7 +6990,12 @@
           <t>SOURCE HAS NO QUERIES - safe to redirect</t>
         </is>
       </c>
-      <c r="M126" s="4" t="inlineStr">
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N126" s="4" t="inlineStr">
         <is>
           <t>Merge + 301.</t>
         </is>
@@ -6409,7 +7040,12 @@
       </c>
       <c r="K127" s="5" t="inlineStr"/>
       <c r="L127" s="4" t="inlineStr"/>
-      <c r="M127" s="4" t="inlineStr">
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N127" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -6446,7 +7082,12 @@
       </c>
       <c r="K128" s="5" t="inlineStr"/>
       <c r="L128" s="4" t="inlineStr"/>
-      <c r="M128" s="4" t="inlineStr">
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N128" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -6491,7 +7132,12 @@
       </c>
       <c r="K129" s="5" t="inlineStr"/>
       <c r="L129" s="4" t="inlineStr"/>
-      <c r="M129" s="4" t="inlineStr">
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N129" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6536,7 +7182,12 @@
       </c>
       <c r="K130" s="5" t="inlineStr"/>
       <c r="L130" s="4" t="inlineStr"/>
-      <c r="M130" s="4" t="inlineStr">
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N130" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6581,7 +7232,12 @@
       </c>
       <c r="K131" s="5" t="inlineStr"/>
       <c r="L131" s="4" t="inlineStr"/>
-      <c r="M131" s="4" t="inlineStr">
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N131" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6626,7 +7282,12 @@
       </c>
       <c r="K132" s="5" t="inlineStr"/>
       <c r="L132" s="4" t="inlineStr"/>
-      <c r="M132" s="4" t="inlineStr">
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N132" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6671,7 +7332,12 @@
       </c>
       <c r="K133" s="5" t="inlineStr"/>
       <c r="L133" s="4" t="inlineStr"/>
-      <c r="M133" s="4" t="inlineStr">
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N133" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6716,7 +7382,12 @@
       </c>
       <c r="K134" s="5" t="inlineStr"/>
       <c r="L134" s="4" t="inlineStr"/>
-      <c r="M134" s="4" t="inlineStr">
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N134" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6761,7 +7432,12 @@
       </c>
       <c r="K135" s="5" t="inlineStr"/>
       <c r="L135" s="4" t="inlineStr"/>
-      <c r="M135" s="4" t="inlineStr">
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N135" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6806,7 +7482,12 @@
       </c>
       <c r="K136" s="5" t="inlineStr"/>
       <c r="L136" s="4" t="inlineStr"/>
-      <c r="M136" s="4" t="inlineStr">
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N136" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6851,7 +7532,12 @@
       </c>
       <c r="K137" s="5" t="inlineStr"/>
       <c r="L137" s="4" t="inlineStr"/>
-      <c r="M137" s="4" t="inlineStr">
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N137" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6896,7 +7582,12 @@
       </c>
       <c r="K138" s="5" t="inlineStr"/>
       <c r="L138" s="4" t="inlineStr"/>
-      <c r="M138" s="4" t="inlineStr">
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N138" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -6941,7 +7632,12 @@
       </c>
       <c r="K139" s="5" t="inlineStr"/>
       <c r="L139" s="4" t="inlineStr"/>
-      <c r="M139" s="4" t="inlineStr">
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N139" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -6986,7 +7682,12 @@
       </c>
       <c r="K140" s="5" t="inlineStr"/>
       <c r="L140" s="4" t="inlineStr"/>
-      <c r="M140" s="4" t="inlineStr">
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N140" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7031,7 +7732,12 @@
       </c>
       <c r="K141" s="5" t="inlineStr"/>
       <c r="L141" s="4" t="inlineStr"/>
-      <c r="M141" s="4" t="inlineStr">
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N141" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -7076,7 +7782,12 @@
       </c>
       <c r="K142" s="5" t="inlineStr"/>
       <c r="L142" s="4" t="inlineStr"/>
-      <c r="M142" s="4" t="inlineStr">
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N142" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -7121,7 +7832,12 @@
       </c>
       <c r="K143" s="5" t="inlineStr"/>
       <c r="L143" s="4" t="inlineStr"/>
-      <c r="M143" s="4" t="inlineStr">
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N143" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -7166,7 +7882,12 @@
       </c>
       <c r="K144" s="5" t="inlineStr"/>
       <c r="L144" s="4" t="inlineStr"/>
-      <c r="M144" s="4" t="inlineStr">
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N144" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7223,7 +7944,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M145" s="4" t="inlineStr">
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N145" s="4" t="inlineStr">
         <is>
           <t>Merge + 301.</t>
         </is>
@@ -7276,7 +8002,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M146" s="4" t="inlineStr">
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N146" s="4" t="inlineStr">
         <is>
           <t>GSC-validated survivor: 75 queries vs 21 on the alternative. Canonical voice-vs-text post.</t>
         </is>
@@ -7321,7 +8052,12 @@
       </c>
       <c r="K147" s="5" t="inlineStr"/>
       <c r="L147" s="4" t="inlineStr"/>
-      <c r="M147" s="4" t="inlineStr">
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N147" s="4" t="inlineStr">
         <is>
           <t>Canonical WL-pricing GUIDE. 46k impressions @0.06% CTR — rewrite title/meta/snippet, add table + CTA to /whitelabel/pricing.</t>
         </is>
@@ -7366,7 +8102,12 @@
       </c>
       <c r="K148" s="5" t="inlineStr"/>
       <c r="L148" s="4" t="inlineStr"/>
-      <c r="M148" s="4" t="inlineStr">
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N148" s="4" t="inlineStr">
         <is>
           <t>Canonical wrapper-vs-native (the "we own the stack" differentiator).</t>
         </is>
@@ -7415,7 +8156,12 @@
       </c>
       <c r="K149" s="5" t="inlineStr"/>
       <c r="L149" s="4" t="inlineStr"/>
-      <c r="M149" s="4" t="inlineStr">
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N149" s="4" t="inlineStr">
         <is>
           <t>Fewer queries (21 vs 75); merge into the stronger page + 301.</t>
         </is>
@@ -7460,7 +8206,12 @@
       </c>
       <c r="K150" s="5" t="inlineStr"/>
       <c r="L150" s="4" t="inlineStr"/>
-      <c r="M150" s="4" t="inlineStr">
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N150" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7505,7 +8256,12 @@
       </c>
       <c r="K151" s="5" t="inlineStr"/>
       <c r="L151" s="4" t="inlineStr"/>
-      <c r="M151" s="4" t="inlineStr">
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N151" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7550,7 +8306,12 @@
       </c>
       <c r="K152" s="5" t="inlineStr"/>
       <c r="L152" s="4" t="inlineStr"/>
-      <c r="M152" s="4" t="inlineStr">
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N152" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7595,7 +8356,12 @@
       </c>
       <c r="K153" s="5" t="inlineStr"/>
       <c r="L153" s="4" t="inlineStr"/>
-      <c r="M153" s="4" t="inlineStr">
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N153" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7640,7 +8406,12 @@
       </c>
       <c r="K154" s="5" t="inlineStr"/>
       <c r="L154" s="4" t="inlineStr"/>
-      <c r="M154" s="4" t="inlineStr">
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N154" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -7697,7 +8468,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M155" s="4" t="inlineStr">
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N155" s="4" t="inlineStr">
         <is>
           <t>Chatbot definitional; 301 to voice.</t>
         </is>
@@ -7742,7 +8518,12 @@
       </c>
       <c r="K156" s="5" t="inlineStr"/>
       <c r="L156" s="4" t="inlineStr"/>
-      <c r="M156" s="4" t="inlineStr">
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N156" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -7787,7 +8568,12 @@
       </c>
       <c r="K157" s="5" t="inlineStr"/>
       <c r="L157" s="4" t="inlineStr"/>
-      <c r="M157" s="4" t="inlineStr">
+      <c r="M157" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N157" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -7832,7 +8618,12 @@
       </c>
       <c r="K158" s="5" t="inlineStr"/>
       <c r="L158" s="4" t="inlineStr"/>
-      <c r="M158" s="4" t="inlineStr">
+      <c r="M158" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N158" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -7877,7 +8668,12 @@
       </c>
       <c r="K159" s="5" t="inlineStr"/>
       <c r="L159" s="4" t="inlineStr"/>
-      <c r="M159" s="4" t="inlineStr">
+      <c r="M159" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N159" s="4" t="inlineStr">
         <is>
           <t>Keep as integrations spoke; link up to /integrations hub.</t>
         </is>
@@ -7934,7 +8730,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M160" s="4" t="inlineStr">
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N160" s="4" t="inlineStr">
         <is>
           <t>Chatbot-framed; 301 to voice pricing guide.</t>
         </is>
@@ -7991,7 +8792,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M161" s="4" t="inlineStr">
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N161" s="4" t="inlineStr">
         <is>
           <t>Merge tool into voice ROI model; 301.</t>
         </is>
@@ -8036,7 +8842,12 @@
       </c>
       <c r="K162" s="5" t="inlineStr"/>
       <c r="L162" s="4" t="inlineStr"/>
-      <c r="M162" s="4" t="inlineStr">
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N162" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8081,7 +8892,12 @@
       </c>
       <c r="K163" s="5" t="inlineStr"/>
       <c r="L163" s="4" t="inlineStr"/>
-      <c r="M163" s="4" t="inlineStr">
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N163" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8126,7 +8942,12 @@
       </c>
       <c r="K164" s="5" t="inlineStr"/>
       <c r="L164" s="4" t="inlineStr"/>
-      <c r="M164" s="4" t="inlineStr">
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N164" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -8171,7 +8992,12 @@
       </c>
       <c r="K165" s="5" t="inlineStr"/>
       <c r="L165" s="4" t="inlineStr"/>
-      <c r="M165" s="4" t="inlineStr">
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N165" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -8216,7 +9042,12 @@
       </c>
       <c r="K166" s="5" t="inlineStr"/>
       <c r="L166" s="4" t="inlineStr"/>
-      <c r="M166" s="4" t="inlineStr">
+      <c r="M166" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N166" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -8261,7 +9092,12 @@
       </c>
       <c r="K167" s="5" t="inlineStr"/>
       <c r="L167" s="4" t="inlineStr"/>
-      <c r="M167" s="4" t="inlineStr">
+      <c r="M167" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N167" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -8306,7 +9142,12 @@
       </c>
       <c r="K168" s="5" t="inlineStr"/>
       <c r="L168" s="4" t="inlineStr"/>
-      <c r="M168" s="4" t="inlineStr">
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N168" s="4" t="inlineStr">
         <is>
           <t>Keep. Link up to /whitelabel + cross-link its /receptionist/industries counterpart (differentiate reseller vs end-customer).</t>
         </is>
@@ -8351,7 +9192,12 @@
       </c>
       <c r="K169" s="5" t="inlineStr"/>
       <c r="L169" s="4" t="inlineStr"/>
-      <c r="M169" s="4" t="inlineStr">
+      <c r="M169" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N169" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8408,7 +9254,12 @@
           <t>MEDIUM - review shared</t>
         </is>
       </c>
-      <c r="M170" s="4" t="inlineStr">
+      <c r="M170" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N170" s="4" t="inlineStr">
         <is>
           <t>Near-duplicate; merge + 301.</t>
         </is>
@@ -8453,7 +9304,12 @@
       </c>
       <c r="K171" s="5" t="inlineStr"/>
       <c r="L171" s="4" t="inlineStr"/>
-      <c r="M171" s="4" t="inlineStr">
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N171" s="4" t="inlineStr">
         <is>
           <t>Canonical profit-margins post.</t>
         </is>
@@ -8498,7 +9354,12 @@
       </c>
       <c r="K172" s="5" t="inlineStr"/>
       <c r="L172" s="4" t="inlineStr"/>
-      <c r="M172" s="4" t="inlineStr">
+      <c r="M172" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N172" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -8543,7 +9404,12 @@
       </c>
       <c r="K173" s="5" t="inlineStr"/>
       <c r="L173" s="4" t="inlineStr"/>
-      <c r="M173" s="4" t="inlineStr">
+      <c r="M173" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N173" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8588,7 +9454,12 @@
       </c>
       <c r="K174" s="5" t="inlineStr"/>
       <c r="L174" s="4" t="inlineStr"/>
-      <c r="M174" s="4" t="inlineStr">
+      <c r="M174" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N174" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8633,7 +9504,12 @@
       </c>
       <c r="K175" s="5" t="inlineStr"/>
       <c r="L175" s="4" t="inlineStr"/>
-      <c r="M175" s="4" t="inlineStr">
+      <c r="M175" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N175" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8678,7 +9554,12 @@
       </c>
       <c r="K176" s="5" t="inlineStr"/>
       <c r="L176" s="4" t="inlineStr"/>
-      <c r="M176" s="4" t="inlineStr">
+      <c r="M176" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N176" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8723,7 +9604,12 @@
       </c>
       <c r="K177" s="5" t="inlineStr"/>
       <c r="L177" s="4" t="inlineStr"/>
-      <c r="M177" s="4" t="inlineStr">
+      <c r="M177" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N177" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8768,7 +9654,12 @@
       </c>
       <c r="K178" s="5" t="inlineStr"/>
       <c r="L178" s="4" t="inlineStr"/>
-      <c r="M178" s="4" t="inlineStr">
+      <c r="M178" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N178" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8825,7 +9716,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M179" s="4" t="inlineStr">
+      <c r="M179" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N179" s="4" t="inlineStr">
         <is>
           <t>Off-topic (chatgpt); 301 to hub.</t>
         </is>
@@ -8870,7 +9766,12 @@
       </c>
       <c r="K180" s="5" t="inlineStr"/>
       <c r="L180" s="4" t="inlineStr"/>
-      <c r="M180" s="4" t="inlineStr">
+      <c r="M180" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N180" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8915,7 +9816,12 @@
       </c>
       <c r="K181" s="5" t="inlineStr"/>
       <c r="L181" s="4" t="inlineStr"/>
-      <c r="M181" s="4" t="inlineStr">
+      <c r="M181" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N181" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -8960,7 +9866,12 @@
       </c>
       <c r="K182" s="5" t="inlineStr"/>
       <c r="L182" s="4" t="inlineStr"/>
-      <c r="M182" s="4" t="inlineStr">
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N182" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -9005,7 +9916,12 @@
       </c>
       <c r="K183" s="5" t="inlineStr"/>
       <c r="L183" s="4" t="inlineStr"/>
-      <c r="M183" s="4" t="inlineStr">
+      <c r="M183" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N183" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -9062,7 +9978,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M184" s="4" t="inlineStr">
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N184" s="4" t="inlineStr">
         <is>
           <t>Merge + 301. SURVIVOR REVIEW: this source has 13 queries vs 2 on the target — confirm which URL survives before 301.</t>
         </is>
@@ -9119,7 +10040,12 @@
           <t>LOW - keep both</t>
         </is>
       </c>
-      <c r="M185" s="4" t="inlineStr">
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N185" s="4" t="inlineStr">
         <is>
           <t>Chatbot build-vs-buy; 301 to canonical build-vs-buy.</t>
         </is>
@@ -9164,7 +10090,12 @@
       </c>
       <c r="K186" s="5" t="inlineStr"/>
       <c r="L186" s="4" t="inlineStr"/>
-      <c r="M186" s="4" t="inlineStr">
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N186" s="4" t="inlineStr">
         <is>
           <t>Distinct intent — keep as spoke; add hub link + related-in-cluster module.</t>
         </is>
@@ -9209,7 +10140,12 @@
       </c>
       <c r="K187" s="5" t="inlineStr"/>
       <c r="L187" s="4" t="inlineStr"/>
-      <c r="M187" s="4" t="inlineStr">
+      <c r="M187" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N187" s="4" t="inlineStr">
         <is>
           <t>Keep. Organise under the Academy hub; link to /partners application.</t>
         </is>
@@ -9254,7 +10190,12 @@
       </c>
       <c r="K188" s="5" t="inlineStr"/>
       <c r="L188" s="4" t="inlineStr"/>
-      <c r="M188" s="4" t="inlineStr">
+      <c r="M188" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N188" s="4" t="inlineStr">
         <is>
           <t>Keep (single competitor/angle). Ensure comparison table, current pricing, compliance wedge, CTA.</t>
         </is>
@@ -9299,7 +10240,12 @@
       </c>
       <c r="K189" s="5" t="inlineStr"/>
       <c r="L189" s="4" t="inlineStr"/>
-      <c r="M189" s="4" t="inlineStr">
+      <c r="M189" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N189" s="4" t="inlineStr">
         <is>
           <t>Revamp under the program hub.</t>
         </is>
@@ -9344,7 +10290,12 @@
       </c>
       <c r="K190" s="5" t="inlineStr"/>
       <c r="L190" s="4" t="inlineStr"/>
-      <c r="M190" s="4" t="inlineStr">
+      <c r="M190" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N190" s="4" t="inlineStr">
         <is>
           <t>Revamp; link from voice-ai-agency-referral-program.</t>
         </is>
@@ -9389,7 +10340,12 @@
       </c>
       <c r="K191" s="5" t="inlineStr"/>
       <c r="L191" s="4" t="inlineStr"/>
-      <c r="M191" s="4" t="inlineStr">
+      <c r="M191" s="2" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="N191" s="4" t="inlineStr">
         <is>
           <t>Revamp under the program hub; wire Academy posts to it.</t>
         </is>
@@ -9438,14 +10394,19 @@
       </c>
       <c r="K192" s="5" t="inlineStr"/>
       <c r="L192" s="4" t="inlineStr"/>
-      <c r="M192" s="4" t="inlineStr">
+      <c r="M192" s="2" t="inlineStr">
+        <is>
+          <t>308 -&gt; https://trillet.ai/whitelabel</t>
+        </is>
+      </c>
+      <c r="N192" s="4" t="inlineStr">
         <is>
           <t>ALREADY 308-redirected to /whitelabel (permanent; passes signal like a 301) - NO ACTION. Its historical head-term impressions in the 16-mo data will consolidate into /whitelabel as Google reprocesses (same as the apex/www fix). Only verify no internal links still point to /agency.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M192"/>
+  <autoFilter ref="A1:N192"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>